<commit_message>
APR armários do supervisório: ajusta local e riscos da atividade principal
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011x7qWfGgJnPkRQ42TgXMmF
</commit_message>
<xml_diff>
--- a/Descarregamento, movimentação e instalação de armários planejados para a sala do supervisório do processo.xlsx
+++ b/Descarregamento, movimentação e instalação de armários planejados para a sala do supervisório do processo.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APR Execução(Modelo) " sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'APR Execução(Modelo) '!$A$1:$R$115</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'APR Execução(Modelo) '!$A$1:$R$97</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -1811,11 +1811,11 @@
   <oneCellAnchor>
     <from>
       <col>15</col>
-      <colOff>1038225</colOff>
+      <colOff>190500</colOff>
       <row>46</row>
-      <rowOff>914400</rowOff>
+      <rowOff>1762125</rowOff>
     </from>
-    <ext cx="2114550" cy="1657350"/>
+    <ext cx="3810000" cy="2286000"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -1836,11 +1836,11 @@
   <oneCellAnchor>
     <from>
       <col>15</col>
-      <colOff>190500</colOff>
-      <row>47</row>
-      <rowOff>504825</rowOff>
+      <colOff>1171575</colOff>
+      <row>64</row>
+      <rowOff>238125</rowOff>
     </from>
-    <ext cx="3810000" cy="2286000"/>
+    <ext cx="1838325" cy="1704975"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -1861,11 +1861,11 @@
   <oneCellAnchor>
     <from>
       <col>15</col>
-      <colOff>1171575</colOff>
-      <row>82</row>
-      <rowOff>238125</rowOff>
+      <colOff>1123950</colOff>
+      <row>64</row>
+      <rowOff>2324100</rowOff>
     </from>
-    <ext cx="1838325" cy="1704975"/>
+    <ext cx="1933575" cy="1543050"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -1873,31 +1873,6 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>15</col>
-      <colOff>1123950</colOff>
-      <row>82</row>
-      <rowOff>2324100</rowOff>
-    </from>
-    <ext cx="1933575" cy="1543050"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2232,7 +2207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T115"/>
+  <dimension ref="A1:T97"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col width="5.28515625" customWidth="1" style="1" min="1" max="1"/>
@@ -2462,7 +2437,7 @@
       <c r="E8" s="260" t="n"/>
       <c r="F8" s="154" t="inlineStr">
         <is>
-          <t>Sala do supervisório do processo – descarregamento próximo ao recebimento de malte (alinhamento do elevador do processo)</t>
+          <t>Sala do supervisório do processo</t>
         </is>
       </c>
       <c r="G8" s="259" t="n"/>
@@ -3034,7 +3009,7 @@
       <c r="E25" s="260" t="n"/>
       <c r="F25" s="154" t="inlineStr">
         <is>
-          <t>Sala do supervisório do processo – descarregamento próximo ao recebimento de malte (alinhamento do elevador do processo)</t>
+          <t>Sala do supervisório do processo</t>
         </is>
       </c>
       <c r="G25" s="259" t="n"/>
@@ -3605,7 +3580,7 @@
       <c r="E42" s="260" t="n"/>
       <c r="F42" s="154" t="inlineStr">
         <is>
-          <t>Sala do supervisório do processo – descarregamento próximo ao recebimento de malte (alinhamento do elevador do processo)</t>
+          <t>Sala do supervisório do processo</t>
         </is>
       </c>
       <c r="G42" s="259" t="n"/>
@@ -3721,7 +3696,7 @@
       <c r="Q46" s="276" t="n"/>
       <c r="R46" s="276" t="n"/>
     </row>
-    <row r="47" ht="267.375" customHeight="1">
+    <row r="47" ht="229.125" customHeight="1">
       <c r="B47" s="152" t="n">
         <v>3</v>
       </c>
@@ -3747,22 +3722,13 @@
       <c r="F47" s="269" t="n"/>
       <c r="G47" s="37" t="inlineStr">
         <is>
-          <t>RISCOS FÍSICOS:
-1. Exposição a ruído
-RISCOS QUÍMICOS:
-2. Poeira de malte na área de descarregamento
-RISCOS ERGONÔMICOS:
-3. Posturas inadequadas
-4. Movimentos repetitivos
+          <t>RISCOS ERGONÔMICOS:
+1. Posturas inadequadas
+2. Movimentos repetitivos
 RISCOS DE ACIDENTES:
-5. Cortes / Prensamento de membros
-6. Projeção de material e de partículas
-7. Batida contra
-8. Queda de pessoas de mesmo nível
-9. Atropelamento
-10. Prensamento / queda de carga no elevador do processo
-11. Tombamento de armários e painéis durante a montagem
-12. Interferência em equipamentos do supervisório em operação</t>
+3. Projeção de material e de partículas
+4. Queda de pessoas de mesmo nível
+5. Queda de materiais</t>
         </is>
       </c>
       <c r="H47" s="228" t="inlineStr">
@@ -3775,33 +3741,31 @@
       <c r="I47" s="277" t="inlineStr">
         <is>
           <t>Acompanhamento Full time responsável Ambev
-Exposição a ruído
-1. Utilizar protetor auricular (tipo plug ou concha) sempre que atuar em ambientes ou operar equipamentos que apresentem níveis elevados de ruído, garantindo a proteção da audição.
-Poeira de malte na área de descarregamento
-2. Alinhar com a operação Ambev para que o descarregamento dos armários não coincida com o descarregamento de malte.
-2.1. Utilizar máscara PFF2 quando houver poeira de malte em suspensão no local do descarregamento.
 Posturas inadequadas
-3. Manter a coluna ereta, evitando curvar excessivamente as costas durante as atividades.
-3.1. Flexionar os joelhos ao abaixar ou levantar cargas, utilizando a força das pernas e não da lombar.
-3.2. Evitar torções do tronco; sempre movimentar o corpo inteiro ao mudar de direção.
-3.3. Ajustar a altura de bancadas, mesas e equipamentos para evitar inclinações prolongadas do corpo.
-3.4. Alternar posturas e realizar pausas periódicas para alongamento e descanso muscular.
-3.5. Evitar permanecer longos períodos na mesma posição, seja em pé, sentado ou agachado.
-3.6. Comunicar imediatamente ao responsável qualquer desconforto, dor ou fadiga, interrompendo a atividade se necessário.
+1. Manter a coluna ereta, evitando curvar excessivamente as costas durante as atividades.
+1.1. Flexionar os joelhos ao abaixar ou levantar cargas, utilizando a força das pernas e não da lombar.
+1.2. Evitar torções do tronco; sempre movimentar o corpo inteiro ao mudar de direção.
+1.3. Ajustar a altura de bancadas, mesas e equipamentos para evitar inclinações prolongadas do corpo.
+1.4. Alternar posturas e realizar pausas periódicas para alongamento e descanso muscular.
+1.5. Evitar permanecer longos períodos na mesma posição, seja em pé, sentado ou agachado.
+1.6. Comunicar imediatamente ao responsável qualquer desconforto, dor ou fadiga, interrompendo a atividade se necessário.
 Movimentos repetitivos
-4. Realizar rodízio de atividades para reduzir a sobrecarga contínua dos mesmos grupos musculares.
-4.1. Utilizar ferramentas mecanizadas, ergonômicas ou auxiliares sempre que possível para diminuir a repetitividade manual.
-4.2. Planejar o ritmo de trabalho, evitando execução acelerada e contínua e movimentos bruscos ou de impacto repetitivo.
-Cortes / Prensamento de membros
-5. Utilizar luvas compatíveis com a atividade (Hyflex / Vaqueta; anticorte no manuseio de chapas e tubos).
-5.1. Manter as mãos e demais membros afastados de partes móveis, áreas de corte e pontos de prensamento.
-5.2. Nunca remover, improvisar ou inutilizar proteções, carenagens e dispositivos de segurança das máquinas e ferramentas.
-5.3. Garantir que máquinas e ferramentas estejam desligadas e desconectadas da energia antes de ajustes, troca de disco, limpezas ou manutenções (ex.: lixadeira).
-5.4. Utilizar ferramentas apropriadas para cada tarefa, evitando o uso das mãos como apoio ou guia.
-5.5. Manter atenção total durante a execução da atividade, evitando distrações.
-5.6. Realizar treinamento NR-12 para operação segura de máquinas e ferramentas.
+2. Realizar rodízio de atividades para reduzir a sobrecarga contínua dos mesmos grupos musculares.
+2.1. Utilizar ferramentas mecanizadas, ergonômicas ou auxiliares sempre que possível para diminuir a repetitividade manual.
+2.2. Planejar o ritmo de trabalho, evitando execução acelerada e contínua e movimentos bruscos ou de impacto repetitivo.
 Projeção de material e de partículas
-6. Fazer uso dos óculos de segurança contra impacto; em caso de lixadeira, fazer o uso do protetor facial.</t>
+3. Fazer uso dos óculos de segurança contra impacto; em caso de lixadeira, fazer o uso do protetor facial.
+Queda de pessoas de mesmo nível
+4. Os colaboradores deverão estar atentos às possíveis interferências existentes no piso.
+4.1. Não correr.
+Queda de materiais
+5. Realizar o posicionamento e o alinhamento dos módulos com no mínimo duas pessoas.
+5.1. Manter os módulos altos apoiados e escorados até a fixação definitiva.
+5.2. Fixar os armários e os painéis de televisão à parede conforme o projeto do fabricante.
+5.3. Não deixar peças, portas e prateleiras soltas apoiadas na vertical sem travamento.
+5.4. Antes de fixar parafusos na parede, verificar com a manutenção Ambev a existência de tubulações e eletrodutos embutidos.
+**Qualquer ocorrência, incidente ou CI deverá ser reportado ao responsável Ambev.
+EM CASO DE EMERGÊNCIA ACIONAR A BRIGADA DE EMERGÊNCIA: 31 98298-4065</t>
         </is>
       </c>
       <c r="J47" s="268" t="n"/>
@@ -3822,7 +3786,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="267.375" customHeight="1">
+    <row r="48" ht="229.125" customHeight="1">
       <c r="B48" s="276" t="n"/>
       <c r="C48" s="273" t="n"/>
       <c r="D48" s="275" t="n"/>
@@ -4221,7 +4185,7 @@
       <c r="E60" s="260" t="n"/>
       <c r="F60" s="154" t="inlineStr">
         <is>
-          <t>Sala do supervisório do processo – descarregamento próximo ao recebimento de malte (alinhamento do elevador do processo)</t>
+          <t>Sala do supervisório do processo</t>
         </is>
       </c>
       <c r="G60" s="259" t="n"/>
@@ -4337,606 +4301,17 @@
       <c r="Q64" s="276" t="n"/>
       <c r="R64" s="276" t="n"/>
     </row>
-    <row r="65" ht="222.75" customHeight="1">
+    <row r="65" ht="330" customHeight="1">
       <c r="B65" s="152" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C65" s="228" t="inlineStr">
         <is>
-          <t>Continuação...</t>
-        </is>
-      </c>
-      <c r="D65" s="269" t="n"/>
+          <t>5S, limpeza e organização da área.</t>
+        </is>
+      </c>
+      <c r="D65" s="260" t="n"/>
       <c r="E65" s="229" t="inlineStr">
-        <is>
-          <t>Continuação</t>
-        </is>
-      </c>
-      <c r="F65" s="269" t="n"/>
-      <c r="G65" s="37" t="inlineStr">
-        <is>
-          <t>Continuação...</t>
-        </is>
-      </c>
-      <c r="H65" s="228" t="inlineStr">
-        <is>
-          <t>Continuação...</t>
-        </is>
-      </c>
-      <c r="I65" s="277" t="inlineStr">
-        <is>
-          <t>Batida contra
-7. Garantir que a área com superfície irregular esteja bem iluminada para facilitar a visualização de obstáculos.
-7.1. Transportar peças longas e volumosas em dupla, com visão livre do trajeto e atenção a portas e corredores até a sala do supervisório.
-Queda de pessoas de mesmo nível
-8. Os colaboradores deverão estar atentos às possíveis interferências existentes no piso.
-8.1. Não correr.
-Atropelamento
-9. Isolar e sinalizar a área de operação do equipamento.
-9.1. Manter somente pessoas autorizadas na área de operação do equipamento.
-9.2. Quando o operador não tiver visão plena da área de operação, utilizar sinaleiro e manter comunicação constante entre operador, sinaleiro e equipe.
-Prensamento / queda de carga no elevador do processo
-10. Utilizar o elevador do processo somente com autorização da operação Ambev.
-10.1. Respeitar a capacidade de carga indicada no elevador; não exceder o limite.
-10.2. Posicionar e apoiar os armários e peças de forma estável no interior do elevador antes do acionamento.
-10.3. Manter mãos e pés afastados das portas do elevador durante a abertura, o fechamento e a movimentação.
-Tombamento de armários e painéis durante a montagem
-11. Realizar o posicionamento e o alinhamento dos módulos com no mínimo duas pessoas.
-11.1. Manter os módulos altos apoiados e escorados até a fixação definitiva.
-11.2. Fixar os armários e os painéis de televisão à parede conforme o projeto do fabricante.
-11.3. Antes de fixar parafusos na parede, verificar com a manutenção Ambev a existência de tubulações e eletrodutos embutidos.
-Interferência em equipamentos do supervisório em operação
-12. Comunicar o operador da sala antes de movimentar peças próximo aos consoles.
-12.1. Proteger consoles, monitores e computadores do supervisório durante a montagem.
-12.2. Não desconectar cabos nem apoiar materiais sobre mesas de operação, painéis e computadores.
-**Qualquer ocorrência, incidente ou CI deverá ser reportado ao responsável Ambev.
-EM CASO DE EMERGÊNCIA ACIONAR A BRIGADA DE EMERGÊNCIA: 31 98298-4065</t>
-        </is>
-      </c>
-      <c r="J65" s="268" t="n"/>
-      <c r="K65" s="268" t="n"/>
-      <c r="L65" s="268" t="n"/>
-      <c r="M65" s="268" t="n"/>
-      <c r="N65" s="268" t="n"/>
-      <c r="O65" s="269" t="n"/>
-      <c r="P65" s="13" t="n"/>
-      <c r="Q65" s="38" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="R65" s="38" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="222.75" customHeight="1">
-      <c r="B66" s="276" t="n"/>
-      <c r="C66" s="273" t="n"/>
-      <c r="D66" s="275" t="n"/>
-      <c r="E66" s="273" t="n"/>
-      <c r="F66" s="275" t="n"/>
-      <c r="G66" s="276" t="n"/>
-      <c r="H66" s="276" t="n"/>
-      <c r="I66" s="273" t="n"/>
-      <c r="J66" s="274" t="n"/>
-      <c r="K66" s="274" t="n"/>
-      <c r="L66" s="274" t="n"/>
-      <c r="M66" s="274" t="n"/>
-      <c r="N66" s="274" t="n"/>
-      <c r="O66" s="275" t="n"/>
-      <c r="P66" s="276" t="n"/>
-      <c r="Q66" s="276" t="n"/>
-      <c r="R66" s="276" t="n"/>
-    </row>
-    <row r="67" ht="47.25" customHeight="1">
-      <c r="B67" s="278" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL DA EMPRESA:</t>
-        </is>
-      </c>
-      <c r="C67" s="255" t="n"/>
-      <c r="D67" s="255" t="n"/>
-      <c r="E67" s="256" t="n"/>
-      <c r="F67" s="279" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL - SEGURANÇA DO TRABALHO EMPRESA</t>
-        </is>
-      </c>
-      <c r="G67" s="255" t="n"/>
-      <c r="H67" s="256" t="n"/>
-      <c r="I67" s="278" t="inlineStr">
-        <is>
-          <t>SEGURANÇA DO TRABALHO AMBEV</t>
-        </is>
-      </c>
-      <c r="J67" s="255" t="n"/>
-      <c r="K67" s="255" t="n"/>
-      <c r="L67" s="255" t="n"/>
-      <c r="M67" s="255" t="n"/>
-      <c r="N67" s="256" t="n"/>
-      <c r="O67" s="278" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL AMBEV PELA ATIVIDADE</t>
-        </is>
-      </c>
-      <c r="P67" s="255" t="n"/>
-      <c r="Q67" s="255" t="n"/>
-      <c r="R67" s="256" t="n"/>
-    </row>
-    <row r="68" ht="35.25" customHeight="1">
-      <c r="B68" s="280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOME: </t>
-        </is>
-      </c>
-      <c r="C68" s="255" t="n"/>
-      <c r="D68" s="255" t="n"/>
-      <c r="E68" s="256" t="n"/>
-      <c r="F68" s="280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOME: </t>
-        </is>
-      </c>
-      <c r="G68" s="255" t="n"/>
-      <c r="H68" s="256" t="n"/>
-      <c r="I68" s="280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOME: </t>
-        </is>
-      </c>
-      <c r="J68" s="255" t="n"/>
-      <c r="K68" s="255" t="n"/>
-      <c r="L68" s="255" t="n"/>
-      <c r="M68" s="255" t="n"/>
-      <c r="N68" s="256" t="n"/>
-      <c r="O68" s="15" t="inlineStr">
-        <is>
-          <t>NOME:</t>
-        </is>
-      </c>
-      <c r="P68" s="16" t="n"/>
-      <c r="Q68" s="16" t="n"/>
-      <c r="R68" s="17" t="n"/>
-    </row>
-    <row r="69" ht="28.5" customHeight="1">
-      <c r="B69" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº documento: </t>
-        </is>
-      </c>
-      <c r="C69" s="16" t="n"/>
-      <c r="D69" s="16" t="n"/>
-      <c r="E69" s="16" t="n"/>
-      <c r="F69" s="280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº documento: </t>
-        </is>
-      </c>
-      <c r="G69" s="255" t="n"/>
-      <c r="H69" s="256" t="n"/>
-      <c r="I69" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº documento: </t>
-        </is>
-      </c>
-      <c r="J69" s="16" t="n"/>
-      <c r="K69" s="16" t="n"/>
-      <c r="L69" s="16" t="n"/>
-      <c r="M69" s="16" t="n"/>
-      <c r="N69" s="17" t="n"/>
-      <c r="O69" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº documento: </t>
-        </is>
-      </c>
-      <c r="P69" s="16" t="n"/>
-      <c r="Q69" s="16" t="n"/>
-      <c r="R69" s="17" t="n"/>
-    </row>
-    <row r="70" ht="24.75" customHeight="1">
-      <c r="B70" s="281" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Contato: </t>
-        </is>
-      </c>
-      <c r="C70" s="282" t="n"/>
-      <c r="D70" s="282" t="n"/>
-      <c r="E70" s="283" t="n"/>
-      <c r="F70" s="284" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Contato: </t>
-        </is>
-      </c>
-      <c r="G70" s="249" t="n"/>
-      <c r="H70" s="250" t="n"/>
-      <c r="I70" s="18" t="inlineStr">
-        <is>
-          <t>Contato:</t>
-        </is>
-      </c>
-      <c r="J70" s="34" t="n"/>
-      <c r="K70" s="19" t="n"/>
-      <c r="L70" s="19" t="n"/>
-      <c r="M70" s="19" t="n"/>
-      <c r="N70" s="20" t="n"/>
-      <c r="O70" s="18" t="inlineStr">
-        <is>
-          <t>Contato:</t>
-        </is>
-      </c>
-      <c r="P70" s="19" t="n"/>
-      <c r="Q70" s="19" t="n"/>
-      <c r="R70" s="20" t="n"/>
-    </row>
-    <row r="71" ht="24" customHeight="1">
-      <c r="B71" s="39" t="inlineStr">
-        <is>
-          <t>Assinatura:</t>
-        </is>
-      </c>
-      <c r="C71" s="259" t="n"/>
-      <c r="D71" s="259" t="n"/>
-      <c r="E71" s="260" t="n"/>
-      <c r="F71" s="39" t="inlineStr">
-        <is>
-          <t>Assinatura:</t>
-        </is>
-      </c>
-      <c r="G71" s="259" t="n"/>
-      <c r="H71" s="260" t="n"/>
-      <c r="I71" s="39" t="inlineStr">
-        <is>
-          <t>Assinatura:</t>
-        </is>
-      </c>
-      <c r="J71" s="259" t="n"/>
-      <c r="K71" s="259" t="n"/>
-      <c r="L71" s="259" t="n"/>
-      <c r="M71" s="259" t="n"/>
-      <c r="N71" s="260" t="n"/>
-      <c r="O71" s="39" t="inlineStr">
-        <is>
-          <t>Assinatura:</t>
-        </is>
-      </c>
-      <c r="P71" s="259" t="n"/>
-      <c r="Q71" s="259" t="n"/>
-      <c r="R71" s="260" t="n"/>
-    </row>
-    <row r="72" ht="21" customHeight="1">
-      <c r="B72" s="248" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TJ MONTAGENS </t>
-        </is>
-      </c>
-      <c r="C72" s="249" t="n"/>
-      <c r="D72" s="249" t="n"/>
-      <c r="E72" s="250" t="n"/>
-      <c r="F72" s="251" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ANEXO 9 - ANÁLISE PRELIMINAR DE RISCOS / DECLARAÇÃO DE MÉTODOS                                                            </t>
-        </is>
-      </c>
-      <c r="G72" s="249" t="n"/>
-      <c r="H72" s="249" t="n"/>
-      <c r="I72" s="249" t="n"/>
-      <c r="J72" s="249" t="n"/>
-      <c r="K72" s="249" t="n"/>
-      <c r="L72" s="249" t="n"/>
-      <c r="M72" s="249" t="n"/>
-      <c r="N72" s="249" t="n"/>
-      <c r="O72" s="249" t="n"/>
-      <c r="P72" s="249" t="n"/>
-      <c r="Q72" s="249" t="n"/>
-      <c r="R72" s="250" t="n"/>
-      <c r="S72" s="2" t="n"/>
-    </row>
-    <row r="73" ht="21" customHeight="1">
-      <c r="B73" s="252" t="n"/>
-      <c r="E73" s="253" t="n"/>
-      <c r="F73" s="254" t="inlineStr">
-        <is>
-          <t>DATA ELABORAÇÃO / EMISSÃO DA APR:</t>
-        </is>
-      </c>
-      <c r="G73" s="255" t="n"/>
-      <c r="H73" s="256" t="n"/>
-      <c r="I73" s="298" t="n">
-        <v>46321</v>
-      </c>
-      <c r="J73" s="249" t="n"/>
-      <c r="K73" s="249" t="n"/>
-      <c r="L73" s="250" t="n"/>
-      <c r="M73" s="3" t="inlineStr">
-        <is>
-          <t>REVISÃO Nº</t>
-        </is>
-      </c>
-      <c r="N73" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O73" s="5" t="inlineStr">
-        <is>
-          <t>DATA:</t>
-        </is>
-      </c>
-      <c r="P73" s="258" t="n"/>
-      <c r="Q73" s="259" t="n"/>
-      <c r="R73" s="260" t="n"/>
-      <c r="S73" s="6" t="n"/>
-    </row>
-    <row r="74" ht="17.1" customHeight="1" thickBot="1">
-      <c r="B74" s="252" t="n"/>
-      <c r="E74" s="253" t="n"/>
-      <c r="F74" s="261" t="inlineStr">
-        <is>
-          <t>DATA PREVISTA DE INÍCIO:</t>
-        </is>
-      </c>
-      <c r="G74" s="255" t="n"/>
-      <c r="H74" s="262" t="n"/>
-      <c r="I74" s="298" t="n">
-        <v>46322</v>
-      </c>
-      <c r="J74" s="249" t="n"/>
-      <c r="K74" s="249" t="n"/>
-      <c r="L74" s="250" t="n"/>
-      <c r="M74" s="7" t="inlineStr">
-        <is>
-          <t>DATA PREVISTA DE TÉRMINO:</t>
-        </is>
-      </c>
-      <c r="N74" s="8" t="n"/>
-      <c r="O74" s="9" t="n"/>
-      <c r="P74" s="299" t="n">
-        <v>46386</v>
-      </c>
-      <c r="Q74" s="10" t="n"/>
-      <c r="R74" s="11" t="n"/>
-      <c r="S74" s="6" t="n"/>
-    </row>
-    <row r="75" ht="30" customHeight="1">
-      <c r="B75" s="99" t="inlineStr">
-        <is>
-          <t>DESCRIÇÃO DOS TRABALHOS:</t>
-        </is>
-      </c>
-      <c r="C75" s="255" t="n"/>
-      <c r="D75" s="255" t="n"/>
-      <c r="E75" s="256" t="n"/>
-      <c r="F75" s="263" t="inlineStr">
-        <is>
-          <t>Descarregamento, movimentação e instalação de armários planejados para a sala do supervisório do processo</t>
-        </is>
-      </c>
-      <c r="G75" s="264" t="n"/>
-      <c r="H75" s="264" t="n"/>
-      <c r="I75" s="264" t="n"/>
-      <c r="J75" s="264" t="n"/>
-      <c r="K75" s="264" t="n"/>
-      <c r="L75" s="264" t="n"/>
-      <c r="M75" s="264" t="n"/>
-      <c r="N75" s="264" t="n"/>
-      <c r="O75" s="264" t="n"/>
-      <c r="P75" s="264" t="n"/>
-      <c r="Q75" s="264" t="n"/>
-      <c r="R75" s="265" t="n"/>
-      <c r="S75" s="6" t="n"/>
-    </row>
-    <row r="76" ht="28.9" customHeight="1">
-      <c r="B76" s="99" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL DA EMPRESA:</t>
-        </is>
-      </c>
-      <c r="C76" s="255" t="n"/>
-      <c r="D76" s="255" t="n"/>
-      <c r="E76" s="256" t="n"/>
-      <c r="F76" s="266" t="inlineStr">
-        <is>
-          <t>FERNANDO ANACLETO SPINOLA</t>
-        </is>
-      </c>
-      <c r="G76" s="249" t="n"/>
-      <c r="H76" s="249" t="n"/>
-      <c r="I76" s="249" t="n"/>
-      <c r="J76" s="250" t="n"/>
-      <c r="K76" s="131" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TELEFONE: </t>
-        </is>
-      </c>
-      <c r="L76" s="250" t="n"/>
-      <c r="M76" s="132" t="inlineStr">
-        <is>
-          <t>37 99841-8785</t>
-        </is>
-      </c>
-      <c r="N76" s="249" t="n"/>
-      <c r="O76" s="249" t="n"/>
-      <c r="P76" s="249" t="n"/>
-      <c r="Q76" s="249" t="n"/>
-      <c r="R76" s="250" t="n"/>
-      <c r="S76" s="6" t="n"/>
-    </row>
-    <row r="77" ht="26.45" customHeight="1">
-      <c r="B77" s="133" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL SEGURANÇA DA EMPRESA:</t>
-        </is>
-      </c>
-      <c r="C77" s="249" t="n"/>
-      <c r="D77" s="249" t="n"/>
-      <c r="E77" s="250" t="n"/>
-      <c r="F77" s="267" t="inlineStr">
-        <is>
-          <t>FERNANDO ANACLETO SPINOLA</t>
-        </is>
-      </c>
-      <c r="G77" s="259" t="n"/>
-      <c r="H77" s="259" t="n"/>
-      <c r="I77" s="259" t="n"/>
-      <c r="J77" s="260" t="n"/>
-      <c r="K77" s="138" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TELEFONE: </t>
-        </is>
-      </c>
-      <c r="L77" s="260" t="n"/>
-      <c r="M77" s="139" t="inlineStr">
-        <is>
-          <t>37 99841-8785</t>
-        </is>
-      </c>
-      <c r="N77" s="259" t="n"/>
-      <c r="O77" s="259" t="n"/>
-      <c r="P77" s="259" t="n"/>
-      <c r="Q77" s="259" t="n"/>
-      <c r="R77" s="260" t="n"/>
-      <c r="S77" s="6" t="n"/>
-    </row>
-    <row r="78" ht="33" customHeight="1">
-      <c r="B78" s="140" t="inlineStr">
-        <is>
-          <t>LOCAL DA ATIVIDADE:</t>
-        </is>
-      </c>
-      <c r="C78" s="259" t="n"/>
-      <c r="D78" s="259" t="n"/>
-      <c r="E78" s="260" t="n"/>
-      <c r="F78" s="154" t="inlineStr">
-        <is>
-          <t>Sala do supervisório do processo – descarregamento próximo ao recebimento de malte (alinhamento do elevador do processo)</t>
-        </is>
-      </c>
-      <c r="G78" s="259" t="n"/>
-      <c r="H78" s="259" t="n"/>
-      <c r="I78" s="259" t="n"/>
-      <c r="J78" s="259" t="n"/>
-      <c r="K78" s="259" t="n"/>
-      <c r="L78" s="259" t="n"/>
-      <c r="M78" s="259" t="n"/>
-      <c r="N78" s="259" t="n"/>
-      <c r="O78" s="259" t="n"/>
-      <c r="P78" s="259" t="n"/>
-      <c r="Q78" s="259" t="n"/>
-      <c r="R78" s="260" t="n"/>
-      <c r="S78" s="6" t="n"/>
-      <c r="T78" s="12" t="n"/>
-    </row>
-    <row r="79" ht="18" customHeight="1">
-      <c r="B79" s="83" t="inlineStr">
-        <is>
-          <t>SEQUÊNCIA DE ATIVIDADES</t>
-        </is>
-      </c>
-      <c r="C79" s="268" t="n"/>
-      <c r="D79" s="269" t="n"/>
-      <c r="E79" s="83" t="inlineStr">
-        <is>
-          <t>QUAIS AS TÉCNICAS / FERRAMENTAS / EQUIPAMENTOS SERÃO USADOS?</t>
-        </is>
-      </c>
-      <c r="F79" s="269" t="n"/>
-      <c r="G79" s="83" t="inlineStr">
-        <is>
-          <t>DESCRIÇÃO DOS RISCOS</t>
-        </is>
-      </c>
-      <c r="H79" s="83" t="inlineStr">
-        <is>
-          <t>Probabilidade de SIFs / Precusor/Potencial/ Real</t>
-        </is>
-      </c>
-      <c r="I79" s="83" t="inlineStr">
-        <is>
-          <t>MEDIDAS DE PRECAUÇÕES E MEDIDAS QUE DEVERÃO SER SEGUIDAS PARA  ELIMINAR OU REDUZIR OS RISCOS.
- (para todos os riscos deve haver uma medida de controle / precaução)</t>
-        </is>
-      </c>
-      <c r="J79" s="268" t="n"/>
-      <c r="K79" s="268" t="n"/>
-      <c r="L79" s="268" t="n"/>
-      <c r="M79" s="268" t="n"/>
-      <c r="N79" s="268" t="n"/>
-      <c r="O79" s="269" t="n"/>
-      <c r="P79" s="83" t="inlineStr">
-        <is>
-          <t>FOTOS ILUSTRATIVA</t>
-        </is>
-      </c>
-      <c r="Q79" s="233" t="inlineStr">
-        <is>
-          <t>Necessidade  de acompanhamento full time  ambev (A/B/C)</t>
-        </is>
-      </c>
-      <c r="R79" s="233" t="inlineStr">
-        <is>
-          <t>Necessário Permissão de Trabalho</t>
-        </is>
-      </c>
-      <c r="S79" s="6" t="n"/>
-    </row>
-    <row r="80" ht="17.1" customHeight="1">
-      <c r="B80" s="270" t="n"/>
-      <c r="D80" s="271" t="n"/>
-      <c r="E80" s="270" t="n"/>
-      <c r="F80" s="271" t="n"/>
-      <c r="G80" s="272" t="n"/>
-      <c r="H80" s="272" t="n"/>
-      <c r="I80" s="270" t="n"/>
-      <c r="O80" s="271" t="n"/>
-      <c r="P80" s="272" t="n"/>
-      <c r="Q80" s="272" t="n"/>
-      <c r="R80" s="272" t="n"/>
-    </row>
-    <row r="81" ht="17.1" customHeight="1">
-      <c r="B81" s="270" t="n"/>
-      <c r="D81" s="271" t="n"/>
-      <c r="E81" s="270" t="n"/>
-      <c r="F81" s="271" t="n"/>
-      <c r="G81" s="272" t="n"/>
-      <c r="H81" s="272" t="n"/>
-      <c r="I81" s="270" t="n"/>
-      <c r="O81" s="271" t="n"/>
-      <c r="P81" s="272" t="n"/>
-      <c r="Q81" s="272" t="n"/>
-      <c r="R81" s="272" t="n"/>
-    </row>
-    <row r="82" ht="35.25" customHeight="1">
-      <c r="B82" s="273" t="n"/>
-      <c r="C82" s="274" t="n"/>
-      <c r="D82" s="275" t="n"/>
-      <c r="E82" s="273" t="n"/>
-      <c r="F82" s="275" t="n"/>
-      <c r="G82" s="276" t="n"/>
-      <c r="H82" s="276" t="n"/>
-      <c r="I82" s="273" t="n"/>
-      <c r="J82" s="274" t="n"/>
-      <c r="K82" s="274" t="n"/>
-      <c r="L82" s="274" t="n"/>
-      <c r="M82" s="274" t="n"/>
-      <c r="N82" s="274" t="n"/>
-      <c r="O82" s="275" t="n"/>
-      <c r="P82" s="276" t="n"/>
-      <c r="Q82" s="276" t="n"/>
-      <c r="R82" s="276" t="n"/>
-    </row>
-    <row r="83" ht="330" customHeight="1">
-      <c r="B83" s="152" t="n">
-        <v>4</v>
-      </c>
-      <c r="C83" s="228" t="inlineStr">
-        <is>
-          <t>5S, limpeza e organização da área.</t>
-        </is>
-      </c>
-      <c r="D83" s="260" t="n"/>
-      <c r="E83" s="229" t="inlineStr">
         <is>
           <t>Técnicas utilizadas:
 Finalizadas as atividades a equipe desmobilizará o isolamento, realizará o 5S na área e se deslocará para o canteiro. A equipe irá utilizar carro de mão plataforma (quatro rodas) para transportar materiais e ferramentas (postes de isolamento, correntes de isolamento), devidamente amarrados, utilizando caminhos seguros e faixas de pedestres. O lixo será segregado para descarte e as ferramentas serão armazenadas no contêiner almoxarifado.
@@ -4944,8 +4319,8 @@
 Carro de mão plataforma, postes de isolamento, correntes de isolamento.</t>
         </is>
       </c>
-      <c r="F83" s="260" t="n"/>
-      <c r="G83" s="37" t="inlineStr">
+      <c r="F65" s="260" t="n"/>
+      <c r="G65" s="37" t="inlineStr">
         <is>
           <t>RISCOS DE ACIDENTE:
 1. Tropeço, escorregão e queda de mesmo nível
@@ -4956,14 +4331,14 @@
 5. Postura inadequada</t>
         </is>
       </c>
-      <c r="H83" s="228" t="inlineStr">
+      <c r="H65" s="228" t="inlineStr">
         <is>
           <t>Precursor - Não
 Potencial - Não
 Real - Não</t>
         </is>
       </c>
-      <c r="I83" s="277" t="inlineStr">
+      <c r="I65" s="277" t="inlineStr">
         <is>
           <t>1. Retirar o isolamento da área (se a atividade não foi finalizada no dia, manter o isolamento);
 1.1. Fazer a limpeza e organização do local, não deixando materiais ou ferramentas desorganizados e fora de locais apropriados;
@@ -4980,918 +4355,936 @@
 EPIs específicos: para manuseio de materiais leves com baixo risco deve-se utilizar luvas multitato. Para manuseio de partes com arestas cortantes, utilizar luvas anticorte ou vaqueta.</t>
         </is>
       </c>
-      <c r="J83" s="259" t="n"/>
-      <c r="K83" s="259" t="n"/>
-      <c r="L83" s="259" t="n"/>
-      <c r="M83" s="259" t="n"/>
-      <c r="N83" s="259" t="n"/>
-      <c r="O83" s="260" t="n"/>
-      <c r="P83" s="13" t="n"/>
-      <c r="Q83" s="38" t="inlineStr">
+      <c r="J65" s="259" t="n"/>
+      <c r="K65" s="259" t="n"/>
+      <c r="L65" s="259" t="n"/>
+      <c r="M65" s="259" t="n"/>
+      <c r="N65" s="259" t="n"/>
+      <c r="O65" s="260" t="n"/>
+      <c r="P65" s="13" t="n"/>
+      <c r="Q65" s="38" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
-      <c r="R83" s="38" t="inlineStr">
+      <c r="R65" s="38" t="inlineStr">
         <is>
           <t>NÃO</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="47.25" customHeight="1">
-      <c r="B84" s="278" t="inlineStr">
+    <row r="66" ht="47.25" customHeight="1">
+      <c r="B66" s="278" t="inlineStr">
         <is>
           <t>RESPONSÁVEL DA EMPRESA:</t>
         </is>
       </c>
+      <c r="C66" s="255" t="n"/>
+      <c r="D66" s="255" t="n"/>
+      <c r="E66" s="256" t="n"/>
+      <c r="F66" s="279" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL - SEGURANÇA DO TRABALHO EMPRESA</t>
+        </is>
+      </c>
+      <c r="G66" s="255" t="n"/>
+      <c r="H66" s="256" t="n"/>
+      <c r="I66" s="278" t="inlineStr">
+        <is>
+          <t>SEGURANÇA DO TRABALHO AMBEV</t>
+        </is>
+      </c>
+      <c r="J66" s="255" t="n"/>
+      <c r="K66" s="255" t="n"/>
+      <c r="L66" s="255" t="n"/>
+      <c r="M66" s="255" t="n"/>
+      <c r="N66" s="256" t="n"/>
+      <c r="O66" s="278" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL AMBEV PELA ATIVIDADE</t>
+        </is>
+      </c>
+      <c r="P66" s="255" t="n"/>
+      <c r="Q66" s="255" t="n"/>
+      <c r="R66" s="256" t="n"/>
+    </row>
+    <row r="67" ht="35.25" customHeight="1">
+      <c r="B67" s="280" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NOME: </t>
+        </is>
+      </c>
+      <c r="C67" s="255" t="n"/>
+      <c r="D67" s="255" t="n"/>
+      <c r="E67" s="256" t="n"/>
+      <c r="F67" s="280" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NOME: </t>
+        </is>
+      </c>
+      <c r="G67" s="255" t="n"/>
+      <c r="H67" s="256" t="n"/>
+      <c r="I67" s="280" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NOME: </t>
+        </is>
+      </c>
+      <c r="J67" s="255" t="n"/>
+      <c r="K67" s="255" t="n"/>
+      <c r="L67" s="255" t="n"/>
+      <c r="M67" s="255" t="n"/>
+      <c r="N67" s="256" t="n"/>
+      <c r="O67" s="15" t="inlineStr">
+        <is>
+          <t>NOME:</t>
+        </is>
+      </c>
+      <c r="P67" s="16" t="n"/>
+      <c r="Q67" s="16" t="n"/>
+      <c r="R67" s="17" t="n"/>
+    </row>
+    <row r="68" ht="28.5" customHeight="1">
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº documento: </t>
+        </is>
+      </c>
+      <c r="C68" s="16" t="n"/>
+      <c r="D68" s="16" t="n"/>
+      <c r="E68" s="16" t="n"/>
+      <c r="F68" s="280" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº documento: </t>
+        </is>
+      </c>
+      <c r="G68" s="255" t="n"/>
+      <c r="H68" s="256" t="n"/>
+      <c r="I68" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº documento: </t>
+        </is>
+      </c>
+      <c r="J68" s="16" t="n"/>
+      <c r="K68" s="16" t="n"/>
+      <c r="L68" s="16" t="n"/>
+      <c r="M68" s="16" t="n"/>
+      <c r="N68" s="17" t="n"/>
+      <c r="O68" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº documento: </t>
+        </is>
+      </c>
+      <c r="P68" s="16" t="n"/>
+      <c r="Q68" s="16" t="n"/>
+      <c r="R68" s="17" t="n"/>
+    </row>
+    <row r="69" ht="24.75" customHeight="1">
+      <c r="B69" s="281" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contato: </t>
+        </is>
+      </c>
+      <c r="C69" s="282" t="n"/>
+      <c r="D69" s="282" t="n"/>
+      <c r="E69" s="283" t="n"/>
+      <c r="F69" s="284" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contato: </t>
+        </is>
+      </c>
+      <c r="G69" s="249" t="n"/>
+      <c r="H69" s="250" t="n"/>
+      <c r="I69" s="18" t="inlineStr">
+        <is>
+          <t>Contato:</t>
+        </is>
+      </c>
+      <c r="J69" s="34" t="n"/>
+      <c r="K69" s="19" t="n"/>
+      <c r="L69" s="19" t="n"/>
+      <c r="M69" s="19" t="n"/>
+      <c r="N69" s="20" t="n"/>
+      <c r="O69" s="18" t="inlineStr">
+        <is>
+          <t>Contato:</t>
+        </is>
+      </c>
+      <c r="P69" s="19" t="n"/>
+      <c r="Q69" s="19" t="n"/>
+      <c r="R69" s="20" t="n"/>
+    </row>
+    <row r="70" ht="24" customHeight="1">
+      <c r="B70" s="39" t="inlineStr">
+        <is>
+          <t>Assinatura:</t>
+        </is>
+      </c>
+      <c r="C70" s="259" t="n"/>
+      <c r="D70" s="259" t="n"/>
+      <c r="E70" s="260" t="n"/>
+      <c r="F70" s="39" t="inlineStr">
+        <is>
+          <t>Assinatura:</t>
+        </is>
+      </c>
+      <c r="G70" s="259" t="n"/>
+      <c r="H70" s="260" t="n"/>
+      <c r="I70" s="39" t="inlineStr">
+        <is>
+          <t>Assinatura:</t>
+        </is>
+      </c>
+      <c r="J70" s="259" t="n"/>
+      <c r="K70" s="259" t="n"/>
+      <c r="L70" s="259" t="n"/>
+      <c r="M70" s="259" t="n"/>
+      <c r="N70" s="260" t="n"/>
+      <c r="O70" s="39" t="inlineStr">
+        <is>
+          <t>Assinatura:</t>
+        </is>
+      </c>
+      <c r="P70" s="259" t="n"/>
+      <c r="Q70" s="259" t="n"/>
+      <c r="R70" s="260" t="n"/>
+    </row>
+    <row r="71" ht="51" customHeight="1">
+      <c r="B71" s="285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TJ MONTAGENS </t>
+        </is>
+      </c>
+      <c r="E71" s="253" t="n"/>
+      <c r="F71" s="214" t="inlineStr">
+        <is>
+          <t>ANEXO 9 - LISTA DE PRESENÇA DO TREINAMENTO DA APR / DECLARAÇÃO DE MÉTODO</t>
+        </is>
+      </c>
+      <c r="S71" s="22" t="n"/>
+      <c r="T71" s="23" t="n"/>
+    </row>
+    <row r="72" hidden="1" ht="408.75" customHeight="1">
+      <c r="B72" s="252" t="n"/>
+      <c r="E72" s="253" t="n"/>
+      <c r="F72" s="286" t="n"/>
+      <c r="G72" s="264" t="n"/>
+      <c r="H72" s="264" t="n"/>
+      <c r="I72" s="264" t="n"/>
+      <c r="J72" s="264" t="n"/>
+      <c r="K72" s="264" t="n"/>
+      <c r="L72" s="264" t="n"/>
+      <c r="M72" s="264" t="n"/>
+      <c r="N72" s="264" t="n"/>
+      <c r="O72" s="264" t="n"/>
+      <c r="P72" s="264" t="n"/>
+      <c r="Q72" s="264" t="n"/>
+      <c r="R72" s="264" t="n"/>
+      <c r="S72" s="24" t="n"/>
+      <c r="T72" s="25" t="n"/>
+    </row>
+    <row r="73" ht="25.5" customHeight="1">
+      <c r="B73" s="286" t="n"/>
+      <c r="C73" s="264" t="n"/>
+      <c r="D73" s="264" t="n"/>
+      <c r="E73" s="265" t="n"/>
+      <c r="F73" s="97" t="inlineStr">
+        <is>
+          <t>DATA PREVISTA DE INÍCIO:</t>
+        </is>
+      </c>
+      <c r="G73" s="256" t="n"/>
+      <c r="H73" s="300" t="n">
+        <v>46322</v>
+      </c>
+      <c r="I73" s="97" t="inlineStr">
+        <is>
+          <t>DATA PREVISTA DE TÉRMINO:</t>
+        </is>
+      </c>
+      <c r="J73" s="255" t="n"/>
+      <c r="K73" s="255" t="n"/>
+      <c r="L73" s="255" t="n"/>
+      <c r="M73" s="255" t="n"/>
+      <c r="N73" s="256" t="n"/>
+      <c r="O73" s="300" t="n">
+        <v>46386</v>
+      </c>
+      <c r="P73" s="255" t="n"/>
+      <c r="Q73" s="255" t="n"/>
+      <c r="R73" s="256" t="n"/>
+      <c r="S73" s="27" t="n"/>
+      <c r="T73" s="28" t="n"/>
+    </row>
+    <row r="74" ht="25.5" customHeight="1" thickBot="1">
+      <c r="B74" s="99" t="inlineStr">
+        <is>
+          <t>DESCRIÇÃO DOS TRABALHOS:</t>
+        </is>
+      </c>
+      <c r="C74" s="255" t="n"/>
+      <c r="D74" s="255" t="n"/>
+      <c r="E74" s="256" t="n"/>
+      <c r="F74" s="146" t="inlineStr">
+        <is>
+          <t>Descarregamento, movimentação e instalação de armários planejados para a sala do supervisório do processo</t>
+        </is>
+      </c>
+      <c r="G74" s="255" t="n"/>
+      <c r="H74" s="255" t="n"/>
+      <c r="I74" s="255" t="n"/>
+      <c r="J74" s="255" t="n"/>
+      <c r="K74" s="255" t="n"/>
+      <c r="L74" s="255" t="n"/>
+      <c r="M74" s="255" t="n"/>
+      <c r="N74" s="255" t="n"/>
+      <c r="O74" s="255" t="n"/>
+      <c r="P74" s="255" t="n"/>
+      <c r="Q74" s="255" t="n"/>
+      <c r="R74" s="255" t="n"/>
+      <c r="S74" s="255" t="n"/>
+      <c r="T74" s="256" t="n"/>
+    </row>
+    <row r="75" ht="22.5" customHeight="1">
+      <c r="B75" s="99" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL DA EMPRESA:</t>
+        </is>
+      </c>
+      <c r="C75" s="255" t="n"/>
+      <c r="D75" s="255" t="n"/>
+      <c r="E75" s="256" t="n"/>
+      <c r="F75" s="147" t="inlineStr">
+        <is>
+          <t>FERNANDO ANACLETO SPINOLA</t>
+        </is>
+      </c>
+      <c r="G75" s="255" t="n"/>
+      <c r="H75" s="255" t="n"/>
+      <c r="I75" s="255" t="n"/>
+      <c r="J75" s="255" t="n"/>
+      <c r="K75" s="255" t="n"/>
+      <c r="L75" s="255" t="n"/>
+      <c r="M75" s="256" t="n"/>
+      <c r="N75" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TELEFONE: </t>
+        </is>
+      </c>
+      <c r="O75" s="256" t="n"/>
+      <c r="P75" s="98" t="inlineStr">
+        <is>
+          <t>37 99841-8785</t>
+        </is>
+      </c>
+      <c r="Q75" s="255" t="n"/>
+      <c r="R75" s="255" t="n"/>
+      <c r="S75" s="255" t="n"/>
+      <c r="T75" s="256" t="n"/>
+    </row>
+    <row r="76" ht="23.25" customHeight="1">
+      <c r="B76" s="99" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL SEGURANÇA DA EMPRESA:</t>
+        </is>
+      </c>
+      <c r="C76" s="255" t="n"/>
+      <c r="D76" s="255" t="n"/>
+      <c r="E76" s="256" t="n"/>
+      <c r="F76" s="205" t="inlineStr">
+        <is>
+          <t>FERNANDO ANACLETO SPINOLA</t>
+        </is>
+      </c>
+      <c r="G76" s="255" t="n"/>
+      <c r="H76" s="255" t="n"/>
+      <c r="I76" s="255" t="n"/>
+      <c r="J76" s="255" t="n"/>
+      <c r="K76" s="255" t="n"/>
+      <c r="L76" s="255" t="n"/>
+      <c r="M76" s="256" t="n"/>
+      <c r="N76" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TELEFONE: </t>
+        </is>
+      </c>
+      <c r="O76" s="256" t="n"/>
+      <c r="P76" s="98" t="inlineStr">
+        <is>
+          <t>37 99841-8785</t>
+        </is>
+      </c>
+      <c r="Q76" s="255" t="n"/>
+      <c r="R76" s="255" t="n"/>
+      <c r="S76" s="255" t="n"/>
+      <c r="T76" s="256" t="n"/>
+    </row>
+    <row r="77" ht="30" customHeight="1">
+      <c r="B77" s="99" t="inlineStr">
+        <is>
+          <t>LOCAL DA ATIVIDADE:</t>
+        </is>
+      </c>
+      <c r="C77" s="255" t="n"/>
+      <c r="D77" s="255" t="n"/>
+      <c r="E77" s="256" t="n"/>
+      <c r="F77" s="147" t="inlineStr">
+        <is>
+          <t>Sala do supervisório do processo</t>
+        </is>
+      </c>
+      <c r="G77" s="255" t="n"/>
+      <c r="H77" s="255" t="n"/>
+      <c r="I77" s="255" t="n"/>
+      <c r="J77" s="255" t="n"/>
+      <c r="K77" s="255" t="n"/>
+      <c r="L77" s="255" t="n"/>
+      <c r="M77" s="255" t="n"/>
+      <c r="N77" s="255" t="n"/>
+      <c r="O77" s="255" t="n"/>
+      <c r="P77" s="255" t="n"/>
+      <c r="Q77" s="255" t="n"/>
+      <c r="R77" s="255" t="n"/>
+      <c r="S77" s="255" t="n"/>
+      <c r="T77" s="256" t="n"/>
+    </row>
+    <row r="78" ht="34.9" customHeight="1">
+      <c r="B78" s="204" t="inlineStr">
+        <is>
+          <t>Declaro que fui treinado e que estou ciente dos riscos e exposições inerentes as atividades que irei executar conforme esta APR / DECLARAÇÃO DE MÉTODOS especificados neste documento.</t>
+        </is>
+      </c>
+      <c r="C78" s="255" t="n"/>
+      <c r="D78" s="255" t="n"/>
+      <c r="E78" s="255" t="n"/>
+      <c r="F78" s="255" t="n"/>
+      <c r="G78" s="255" t="n"/>
+      <c r="H78" s="255" t="n"/>
+      <c r="I78" s="255" t="n"/>
+      <c r="J78" s="255" t="n"/>
+      <c r="K78" s="255" t="n"/>
+      <c r="L78" s="255" t="n"/>
+      <c r="M78" s="255" t="n"/>
+      <c r="N78" s="255" t="n"/>
+      <c r="O78" s="255" t="n"/>
+      <c r="P78" s="255" t="n"/>
+      <c r="Q78" s="255" t="n"/>
+      <c r="R78" s="255" t="n"/>
+      <c r="S78" s="255" t="n"/>
+      <c r="T78" s="256" t="n"/>
+    </row>
+    <row r="79" ht="16.5" customHeight="1">
+      <c r="B79" s="145" t="inlineStr">
+        <is>
+          <t>NOME</t>
+        </is>
+      </c>
+      <c r="C79" s="255" t="n"/>
+      <c r="D79" s="255" t="n"/>
+      <c r="E79" s="256" t="n"/>
+      <c r="F79" s="145" t="inlineStr">
+        <is>
+          <t>CARGO</t>
+        </is>
+      </c>
+      <c r="G79" s="255" t="n"/>
+      <c r="H79" s="256" t="n"/>
+      <c r="I79" s="145" t="inlineStr">
+        <is>
+          <t>ASSINATURA</t>
+        </is>
+      </c>
+      <c r="J79" s="255" t="n"/>
+      <c r="K79" s="255" t="n"/>
+      <c r="L79" s="255" t="n"/>
+      <c r="M79" s="255" t="n"/>
+      <c r="N79" s="255" t="n"/>
+      <c r="O79" s="255" t="n"/>
+      <c r="P79" s="256" t="n"/>
+      <c r="Q79" s="145" t="inlineStr">
+        <is>
+          <t>DATA</t>
+        </is>
+      </c>
+      <c r="R79" s="256" t="n"/>
+      <c r="S79" s="145" t="n"/>
+      <c r="T79" s="256" t="n"/>
+    </row>
+    <row r="80" ht="40.15" customHeight="1">
+      <c r="B80" s="144" t="n"/>
+      <c r="C80" s="255" t="n"/>
+      <c r="D80" s="255" t="n"/>
+      <c r="E80" s="256" t="n"/>
+      <c r="F80" s="144" t="n"/>
+      <c r="G80" s="255" t="n"/>
+      <c r="H80" s="256" t="n"/>
+      <c r="I80" s="144" t="n"/>
+      <c r="J80" s="255" t="n"/>
+      <c r="K80" s="255" t="n"/>
+      <c r="L80" s="255" t="n"/>
+      <c r="M80" s="255" t="n"/>
+      <c r="N80" s="255" t="n"/>
+      <c r="O80" s="255" t="n"/>
+      <c r="P80" s="256" t="n"/>
+      <c r="Q80" s="144" t="n"/>
+      <c r="R80" s="256" t="n"/>
+      <c r="S80" s="144" t="n"/>
+      <c r="T80" s="256" t="n"/>
+    </row>
+    <row r="81" ht="40.15" customHeight="1">
+      <c r="B81" s="144" t="n"/>
+      <c r="C81" s="255" t="n"/>
+      <c r="D81" s="255" t="n"/>
+      <c r="E81" s="256" t="n"/>
+      <c r="F81" s="144" t="n"/>
+      <c r="G81" s="255" t="n"/>
+      <c r="H81" s="256" t="n"/>
+      <c r="I81" s="144" t="n"/>
+      <c r="J81" s="255" t="n"/>
+      <c r="K81" s="255" t="n"/>
+      <c r="L81" s="255" t="n"/>
+      <c r="M81" s="255" t="n"/>
+      <c r="N81" s="255" t="n"/>
+      <c r="O81" s="255" t="n"/>
+      <c r="P81" s="256" t="n"/>
+      <c r="Q81" s="144" t="n"/>
+      <c r="R81" s="256" t="n"/>
+      <c r="S81" s="144" t="n"/>
+      <c r="T81" s="256" t="n"/>
+    </row>
+    <row r="82" ht="40.15" customHeight="1">
+      <c r="B82" s="144" t="n"/>
+      <c r="C82" s="255" t="n"/>
+      <c r="D82" s="255" t="n"/>
+      <c r="E82" s="256" t="n"/>
+      <c r="F82" s="144" t="n"/>
+      <c r="G82" s="255" t="n"/>
+      <c r="H82" s="256" t="n"/>
+      <c r="I82" s="144" t="n"/>
+      <c r="J82" s="255" t="n"/>
+      <c r="K82" s="255" t="n"/>
+      <c r="L82" s="255" t="n"/>
+      <c r="M82" s="255" t="n"/>
+      <c r="N82" s="255" t="n"/>
+      <c r="O82" s="255" t="n"/>
+      <c r="P82" s="256" t="n"/>
+      <c r="Q82" s="144" t="n"/>
+      <c r="R82" s="256" t="n"/>
+      <c r="S82" s="144" t="n"/>
+      <c r="T82" s="256" t="n"/>
+    </row>
+    <row r="83" ht="40.15" customHeight="1">
+      <c r="B83" s="144" t="n"/>
+      <c r="C83" s="255" t="n"/>
+      <c r="D83" s="255" t="n"/>
+      <c r="E83" s="256" t="n"/>
+      <c r="F83" s="144" t="n"/>
+      <c r="G83" s="255" t="n"/>
+      <c r="H83" s="256" t="n"/>
+      <c r="I83" s="144" t="n"/>
+      <c r="J83" s="255" t="n"/>
+      <c r="K83" s="255" t="n"/>
+      <c r="L83" s="255" t="n"/>
+      <c r="M83" s="255" t="n"/>
+      <c r="N83" s="255" t="n"/>
+      <c r="O83" s="255" t="n"/>
+      <c r="P83" s="256" t="n"/>
+      <c r="Q83" s="144" t="n"/>
+      <c r="R83" s="256" t="n"/>
+      <c r="S83" s="144" t="n"/>
+      <c r="T83" s="256" t="n"/>
+    </row>
+    <row r="84" ht="40.15" customHeight="1">
+      <c r="B84" s="144" t="n"/>
       <c r="C84" s="255" t="n"/>
       <c r="D84" s="255" t="n"/>
       <c r="E84" s="256" t="n"/>
-      <c r="F84" s="279" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL - SEGURANÇA DO TRABALHO EMPRESA</t>
-        </is>
-      </c>
+      <c r="F84" s="144" t="n"/>
       <c r="G84" s="255" t="n"/>
       <c r="H84" s="256" t="n"/>
-      <c r="I84" s="278" t="inlineStr">
-        <is>
-          <t>SEGURANÇA DO TRABALHO AMBEV</t>
-        </is>
-      </c>
+      <c r="I84" s="144" t="n"/>
       <c r="J84" s="255" t="n"/>
       <c r="K84" s="255" t="n"/>
       <c r="L84" s="255" t="n"/>
       <c r="M84" s="255" t="n"/>
-      <c r="N84" s="256" t="n"/>
-      <c r="O84" s="278" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL AMBEV PELA ATIVIDADE</t>
-        </is>
-      </c>
-      <c r="P84" s="255" t="n"/>
-      <c r="Q84" s="255" t="n"/>
+      <c r="N84" s="255" t="n"/>
+      <c r="O84" s="255" t="n"/>
+      <c r="P84" s="256" t="n"/>
+      <c r="Q84" s="144" t="n"/>
       <c r="R84" s="256" t="n"/>
-    </row>
-    <row r="85" ht="35.25" customHeight="1">
-      <c r="B85" s="280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOME: </t>
-        </is>
-      </c>
+      <c r="S84" s="144" t="n"/>
+      <c r="T84" s="256" t="n"/>
+    </row>
+    <row r="85" ht="40.15" customHeight="1">
+      <c r="B85" s="144" t="n"/>
       <c r="C85" s="255" t="n"/>
       <c r="D85" s="255" t="n"/>
       <c r="E85" s="256" t="n"/>
-      <c r="F85" s="280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOME: </t>
-        </is>
-      </c>
+      <c r="F85" s="144" t="n"/>
       <c r="G85" s="255" t="n"/>
       <c r="H85" s="256" t="n"/>
-      <c r="I85" s="280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOME: </t>
-        </is>
-      </c>
+      <c r="I85" s="144" t="n"/>
       <c r="J85" s="255" t="n"/>
       <c r="K85" s="255" t="n"/>
       <c r="L85" s="255" t="n"/>
       <c r="M85" s="255" t="n"/>
-      <c r="N85" s="256" t="n"/>
-      <c r="O85" s="15" t="inlineStr">
-        <is>
-          <t>NOME:</t>
-        </is>
-      </c>
-      <c r="P85" s="16" t="n"/>
-      <c r="Q85" s="16" t="n"/>
-      <c r="R85" s="17" t="n"/>
-    </row>
-    <row r="86" ht="28.5" customHeight="1">
-      <c r="B86" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº documento: </t>
-        </is>
-      </c>
-      <c r="C86" s="16" t="n"/>
-      <c r="D86" s="16" t="n"/>
-      <c r="E86" s="16" t="n"/>
-      <c r="F86" s="280" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº documento: </t>
-        </is>
-      </c>
+      <c r="N85" s="255" t="n"/>
+      <c r="O85" s="255" t="n"/>
+      <c r="P85" s="256" t="n"/>
+      <c r="Q85" s="144" t="n"/>
+      <c r="R85" s="256" t="n"/>
+      <c r="S85" s="144" t="n"/>
+      <c r="T85" s="256" t="n"/>
+    </row>
+    <row r="86" ht="40.15" customHeight="1">
+      <c r="B86" s="144" t="n"/>
+      <c r="C86" s="255" t="n"/>
+      <c r="D86" s="255" t="n"/>
+      <c r="E86" s="256" t="n"/>
+      <c r="F86" s="144" t="n"/>
       <c r="G86" s="255" t="n"/>
       <c r="H86" s="256" t="n"/>
-      <c r="I86" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº documento: </t>
-        </is>
-      </c>
-      <c r="J86" s="16" t="n"/>
-      <c r="K86" s="16" t="n"/>
-      <c r="L86" s="16" t="n"/>
-      <c r="M86" s="16" t="n"/>
-      <c r="N86" s="17" t="n"/>
-      <c r="O86" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº documento: </t>
-        </is>
-      </c>
-      <c r="P86" s="16" t="n"/>
-      <c r="Q86" s="16" t="n"/>
-      <c r="R86" s="17" t="n"/>
-    </row>
-    <row r="87" ht="24.75" customHeight="1">
-      <c r="B87" s="281" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Contato: </t>
-        </is>
-      </c>
-      <c r="C87" s="282" t="n"/>
-      <c r="D87" s="282" t="n"/>
-      <c r="E87" s="283" t="n"/>
-      <c r="F87" s="284" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Contato: </t>
-        </is>
-      </c>
-      <c r="G87" s="249" t="n"/>
-      <c r="H87" s="250" t="n"/>
-      <c r="I87" s="18" t="inlineStr">
-        <is>
-          <t>Contato:</t>
-        </is>
-      </c>
-      <c r="J87" s="34" t="n"/>
-      <c r="K87" s="19" t="n"/>
-      <c r="L87" s="19" t="n"/>
-      <c r="M87" s="19" t="n"/>
-      <c r="N87" s="20" t="n"/>
-      <c r="O87" s="18" t="inlineStr">
-        <is>
-          <t>Contato:</t>
-        </is>
-      </c>
-      <c r="P87" s="19" t="n"/>
-      <c r="Q87" s="19" t="n"/>
-      <c r="R87" s="20" t="n"/>
-    </row>
-    <row r="88" ht="24" customHeight="1">
-      <c r="B88" s="39" t="inlineStr">
-        <is>
-          <t>Assinatura:</t>
-        </is>
-      </c>
-      <c r="C88" s="259" t="n"/>
-      <c r="D88" s="259" t="n"/>
-      <c r="E88" s="260" t="n"/>
-      <c r="F88" s="39" t="inlineStr">
-        <is>
-          <t>Assinatura:</t>
-        </is>
-      </c>
-      <c r="G88" s="259" t="n"/>
-      <c r="H88" s="260" t="n"/>
-      <c r="I88" s="39" t="inlineStr">
-        <is>
-          <t>Assinatura:</t>
-        </is>
-      </c>
-      <c r="J88" s="259" t="n"/>
-      <c r="K88" s="259" t="n"/>
-      <c r="L88" s="259" t="n"/>
-      <c r="M88" s="259" t="n"/>
-      <c r="N88" s="260" t="n"/>
-      <c r="O88" s="39" t="inlineStr">
-        <is>
-          <t>Assinatura:</t>
-        </is>
-      </c>
-      <c r="P88" s="259" t="n"/>
-      <c r="Q88" s="259" t="n"/>
-      <c r="R88" s="260" t="n"/>
-    </row>
-    <row r="89" ht="51" customHeight="1">
-      <c r="B89" s="285" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TJ MONTAGENS </t>
-        </is>
-      </c>
-      <c r="E89" s="253" t="n"/>
-      <c r="F89" s="214" t="inlineStr">
-        <is>
-          <t>ANEXO 9 - LISTA DE PRESENÇA DO TREINAMENTO DA APR / DECLARAÇÃO DE MÉTODO</t>
-        </is>
-      </c>
-      <c r="S89" s="22" t="n"/>
-      <c r="T89" s="23" t="n"/>
-    </row>
-    <row r="90" hidden="1" ht="408.75" customHeight="1">
-      <c r="B90" s="252" t="n"/>
-      <c r="E90" s="253" t="n"/>
-      <c r="F90" s="286" t="n"/>
-      <c r="G90" s="264" t="n"/>
-      <c r="H90" s="264" t="n"/>
-      <c r="I90" s="264" t="n"/>
-      <c r="J90" s="264" t="n"/>
-      <c r="K90" s="264" t="n"/>
-      <c r="L90" s="264" t="n"/>
-      <c r="M90" s="264" t="n"/>
-      <c r="N90" s="264" t="n"/>
-      <c r="O90" s="264" t="n"/>
-      <c r="P90" s="264" t="n"/>
-      <c r="Q90" s="264" t="n"/>
-      <c r="R90" s="264" t="n"/>
-      <c r="S90" s="24" t="n"/>
-      <c r="T90" s="25" t="n"/>
-    </row>
-    <row r="91" ht="25.5" customHeight="1">
-      <c r="B91" s="286" t="n"/>
-      <c r="C91" s="264" t="n"/>
-      <c r="D91" s="264" t="n"/>
-      <c r="E91" s="265" t="n"/>
-      <c r="F91" s="97" t="inlineStr">
-        <is>
-          <t>DATA PREVISTA DE INÍCIO:</t>
-        </is>
-      </c>
-      <c r="G91" s="256" t="n"/>
-      <c r="H91" s="300" t="n">
-        <v>46322</v>
-      </c>
-      <c r="I91" s="97" t="inlineStr">
-        <is>
-          <t>DATA PREVISTA DE TÉRMINO:</t>
-        </is>
-      </c>
+      <c r="I86" s="144" t="n"/>
+      <c r="J86" s="255" t="n"/>
+      <c r="K86" s="255" t="n"/>
+      <c r="L86" s="255" t="n"/>
+      <c r="M86" s="255" t="n"/>
+      <c r="N86" s="255" t="n"/>
+      <c r="O86" s="255" t="n"/>
+      <c r="P86" s="256" t="n"/>
+      <c r="Q86" s="144" t="n"/>
+      <c r="R86" s="256" t="n"/>
+      <c r="S86" s="144" t="n"/>
+      <c r="T86" s="256" t="n"/>
+    </row>
+    <row r="87" ht="40.15" customHeight="1">
+      <c r="B87" s="144" t="n"/>
+      <c r="C87" s="255" t="n"/>
+      <c r="D87" s="255" t="n"/>
+      <c r="E87" s="256" t="n"/>
+      <c r="F87" s="144" t="n"/>
+      <c r="G87" s="255" t="n"/>
+      <c r="H87" s="256" t="n"/>
+      <c r="I87" s="144" t="n"/>
+      <c r="J87" s="255" t="n"/>
+      <c r="K87" s="255" t="n"/>
+      <c r="L87" s="255" t="n"/>
+      <c r="M87" s="255" t="n"/>
+      <c r="N87" s="255" t="n"/>
+      <c r="O87" s="255" t="n"/>
+      <c r="P87" s="256" t="n"/>
+      <c r="Q87" s="144" t="n"/>
+      <c r="R87" s="256" t="n"/>
+      <c r="S87" s="144" t="n"/>
+      <c r="T87" s="144" t="n"/>
+    </row>
+    <row r="88" ht="40.15" customHeight="1">
+      <c r="B88" s="144" t="n"/>
+      <c r="C88" s="255" t="n"/>
+      <c r="D88" s="255" t="n"/>
+      <c r="E88" s="256" t="n"/>
+      <c r="F88" s="144" t="n"/>
+      <c r="G88" s="255" t="n"/>
+      <c r="H88" s="256" t="n"/>
+      <c r="I88" s="144" t="n"/>
+      <c r="J88" s="255" t="n"/>
+      <c r="K88" s="255" t="n"/>
+      <c r="L88" s="255" t="n"/>
+      <c r="M88" s="255" t="n"/>
+      <c r="N88" s="255" t="n"/>
+      <c r="O88" s="255" t="n"/>
+      <c r="P88" s="256" t="n"/>
+      <c r="Q88" s="144" t="n"/>
+      <c r="R88" s="256" t="n"/>
+      <c r="S88" s="144" t="n"/>
+      <c r="T88" s="144" t="n"/>
+    </row>
+    <row r="89" ht="40.15" customHeight="1">
+      <c r="B89" s="144" t="n"/>
+      <c r="C89" s="255" t="n"/>
+      <c r="D89" s="255" t="n"/>
+      <c r="E89" s="256" t="n"/>
+      <c r="F89" s="144" t="n"/>
+      <c r="G89" s="255" t="n"/>
+      <c r="H89" s="256" t="n"/>
+      <c r="I89" s="144" t="n"/>
+      <c r="J89" s="255" t="n"/>
+      <c r="K89" s="255" t="n"/>
+      <c r="L89" s="255" t="n"/>
+      <c r="M89" s="255" t="n"/>
+      <c r="N89" s="255" t="n"/>
+      <c r="O89" s="255" t="n"/>
+      <c r="P89" s="256" t="n"/>
+      <c r="Q89" s="144" t="n"/>
+      <c r="R89" s="256" t="n"/>
+      <c r="S89" s="144" t="n"/>
+      <c r="T89" s="144" t="n"/>
+    </row>
+    <row r="90" ht="40.15" customHeight="1">
+      <c r="B90" s="144" t="n"/>
+      <c r="C90" s="255" t="n"/>
+      <c r="D90" s="255" t="n"/>
+      <c r="E90" s="256" t="n"/>
+      <c r="F90" s="144" t="n"/>
+      <c r="G90" s="255" t="n"/>
+      <c r="H90" s="256" t="n"/>
+      <c r="I90" s="144" t="n"/>
+      <c r="J90" s="255" t="n"/>
+      <c r="K90" s="255" t="n"/>
+      <c r="L90" s="255" t="n"/>
+      <c r="M90" s="255" t="n"/>
+      <c r="N90" s="255" t="n"/>
+      <c r="O90" s="255" t="n"/>
+      <c r="P90" s="256" t="n"/>
+      <c r="Q90" s="144" t="n"/>
+      <c r="R90" s="256" t="n"/>
+      <c r="S90" s="144" t="n"/>
+      <c r="T90" s="144" t="n"/>
+    </row>
+    <row r="91" ht="40.15" customHeight="1">
+      <c r="B91" s="144" t="n"/>
+      <c r="C91" s="255" t="n"/>
+      <c r="D91" s="255" t="n"/>
+      <c r="E91" s="256" t="n"/>
+      <c r="F91" s="144" t="n"/>
+      <c r="G91" s="255" t="n"/>
+      <c r="H91" s="256" t="n"/>
+      <c r="I91" s="144" t="n"/>
       <c r="J91" s="255" t="n"/>
       <c r="K91" s="255" t="n"/>
       <c r="L91" s="255" t="n"/>
       <c r="M91" s="255" t="n"/>
-      <c r="N91" s="256" t="n"/>
-      <c r="O91" s="300" t="n">
-        <v>46386</v>
-      </c>
-      <c r="P91" s="255" t="n"/>
-      <c r="Q91" s="255" t="n"/>
+      <c r="N91" s="255" t="n"/>
+      <c r="O91" s="255" t="n"/>
+      <c r="P91" s="256" t="n"/>
+      <c r="Q91" s="144" t="n"/>
       <c r="R91" s="256" t="n"/>
-      <c r="S91" s="27" t="n"/>
-      <c r="T91" s="28" t="n"/>
-    </row>
-    <row r="92" ht="25.5" customHeight="1">
-      <c r="B92" s="99" t="inlineStr">
-        <is>
-          <t>DESCRIÇÃO DOS TRABALHOS:</t>
-        </is>
-      </c>
+      <c r="S91" s="144" t="n"/>
+      <c r="T91" s="144" t="n"/>
+    </row>
+    <row r="92" ht="40.15" customHeight="1">
+      <c r="B92" s="144" t="n"/>
       <c r="C92" s="255" t="n"/>
       <c r="D92" s="255" t="n"/>
       <c r="E92" s="256" t="n"/>
-      <c r="F92" s="146" t="inlineStr">
-        <is>
-          <t>Descarregamento, movimentação e instalação de armários planejados para a sala do supervisório do processo</t>
-        </is>
-      </c>
+      <c r="F92" s="144" t="n"/>
       <c r="G92" s="255" t="n"/>
-      <c r="H92" s="255" t="n"/>
-      <c r="I92" s="255" t="n"/>
+      <c r="H92" s="256" t="n"/>
+      <c r="I92" s="144" t="n"/>
       <c r="J92" s="255" t="n"/>
       <c r="K92" s="255" t="n"/>
       <c r="L92" s="255" t="n"/>
       <c r="M92" s="255" t="n"/>
       <c r="N92" s="255" t="n"/>
       <c r="O92" s="255" t="n"/>
-      <c r="P92" s="255" t="n"/>
-      <c r="Q92" s="255" t="n"/>
-      <c r="R92" s="255" t="n"/>
-      <c r="S92" s="255" t="n"/>
-      <c r="T92" s="256" t="n"/>
-    </row>
-    <row r="93" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B93" s="99" t="inlineStr">
+      <c r="P92" s="256" t="n"/>
+      <c r="Q92" s="144" t="n"/>
+      <c r="R92" s="256" t="n"/>
+      <c r="S92" s="144" t="n"/>
+      <c r="T92" s="144" t="n"/>
+    </row>
+    <row r="93" ht="63.75" customHeight="1" thickBot="1">
+      <c r="B93" s="287" t="inlineStr">
         <is>
           <t>RESPONSÁVEL DA EMPRESA:</t>
         </is>
       </c>
-      <c r="C93" s="255" t="n"/>
-      <c r="D93" s="255" t="n"/>
-      <c r="E93" s="256" t="n"/>
-      <c r="F93" s="147" t="inlineStr">
-        <is>
-          <t>FERNANDO ANACLETO SPINOLA</t>
-        </is>
-      </c>
-      <c r="G93" s="255" t="n"/>
-      <c r="H93" s="255" t="n"/>
-      <c r="I93" s="255" t="n"/>
+      <c r="C93" s="282" t="n"/>
+      <c r="D93" s="282" t="n"/>
+      <c r="E93" s="282" t="n"/>
+      <c r="F93" s="288" t="n"/>
+      <c r="G93" s="197" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL - SEGURANÇA DO TRABALHO EMPRESA</t>
+        </is>
+      </c>
+      <c r="H93" s="256" t="n"/>
+      <c r="I93" s="197" t="inlineStr">
+        <is>
+          <t>SEGURANÇA DO TRABALHO AMBEV</t>
+        </is>
+      </c>
       <c r="J93" s="255" t="n"/>
       <c r="K93" s="255" t="n"/>
       <c r="L93" s="255" t="n"/>
-      <c r="M93" s="256" t="n"/>
-      <c r="N93" s="97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TELEFONE: </t>
-        </is>
-      </c>
-      <c r="O93" s="256" t="n"/>
-      <c r="P93" s="98" t="inlineStr">
-        <is>
-          <t>37 99841-8785</t>
-        </is>
-      </c>
-      <c r="Q93" s="255" t="n"/>
-      <c r="R93" s="255" t="n"/>
-      <c r="S93" s="255" t="n"/>
-      <c r="T93" s="256" t="n"/>
-    </row>
-    <row r="94" ht="23.25" customHeight="1">
-      <c r="B94" s="99" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL SEGURANÇA DA EMPRESA:</t>
-        </is>
-      </c>
-      <c r="C94" s="255" t="n"/>
-      <c r="D94" s="255" t="n"/>
-      <c r="E94" s="256" t="n"/>
-      <c r="F94" s="205" t="inlineStr">
-        <is>
-          <t>FERNANDO ANACLETO SPINOLA</t>
-        </is>
-      </c>
-      <c r="G94" s="255" t="n"/>
-      <c r="H94" s="255" t="n"/>
-      <c r="I94" s="255" t="n"/>
-      <c r="J94" s="255" t="n"/>
-      <c r="K94" s="255" t="n"/>
-      <c r="L94" s="255" t="n"/>
-      <c r="M94" s="256" t="n"/>
-      <c r="N94" s="97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TELEFONE: </t>
-        </is>
-      </c>
-      <c r="O94" s="256" t="n"/>
-      <c r="P94" s="98" t="inlineStr">
-        <is>
-          <t>37 99841-8785</t>
-        </is>
-      </c>
-      <c r="Q94" s="255" t="n"/>
-      <c r="R94" s="255" t="n"/>
-      <c r="S94" s="255" t="n"/>
-      <c r="T94" s="256" t="n"/>
-    </row>
-    <row r="95" ht="30" customHeight="1">
-      <c r="B95" s="99" t="inlineStr">
-        <is>
-          <t>LOCAL DA ATIVIDADE:</t>
-        </is>
-      </c>
-      <c r="C95" s="255" t="n"/>
-      <c r="D95" s="255" t="n"/>
-      <c r="E95" s="256" t="n"/>
-      <c r="F95" s="147" t="inlineStr">
-        <is>
-          <t>Sala do supervisório do processo – descarregamento próximo ao recebimento de malte (alinhamento do elevador do processo)</t>
-        </is>
-      </c>
-      <c r="G95" s="255" t="n"/>
-      <c r="H95" s="255" t="n"/>
-      <c r="I95" s="255" t="n"/>
+      <c r="M93" s="255" t="n"/>
+      <c r="N93" s="256" t="n"/>
+      <c r="O93" s="289" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL AMBEV PELA ATIVIDADE</t>
+        </is>
+      </c>
+      <c r="P93" s="282" t="n"/>
+      <c r="Q93" s="282" t="n"/>
+      <c r="R93" s="283" t="n"/>
+      <c r="S93" s="33" t="n"/>
+      <c r="T93" s="33" t="n"/>
+    </row>
+    <row r="94" ht="37.15" customHeight="1">
+      <c r="B94" s="290" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nome: </t>
+        </is>
+      </c>
+      <c r="C94" s="259" t="n"/>
+      <c r="D94" s="259" t="n"/>
+      <c r="E94" s="259" t="n"/>
+      <c r="F94" s="260" t="n"/>
+      <c r="G94" s="291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nome: </t>
+        </is>
+      </c>
+      <c r="H94" s="260" t="n"/>
+      <c r="I94" s="291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nome: </t>
+        </is>
+      </c>
+      <c r="J94" s="259" t="n"/>
+      <c r="K94" s="259" t="n"/>
+      <c r="L94" s="259" t="n"/>
+      <c r="M94" s="259" t="n"/>
+      <c r="N94" s="260" t="n"/>
+      <c r="O94" s="292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nome: </t>
+        </is>
+      </c>
+      <c r="P94" s="259" t="n"/>
+      <c r="Q94" s="259" t="n"/>
+      <c r="R94" s="259" t="n"/>
+      <c r="S94" s="259" t="n"/>
+      <c r="T94" s="293" t="n"/>
+    </row>
+    <row r="95" ht="38.65" customHeight="1">
+      <c r="B95" s="294" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº documento: </t>
+        </is>
+      </c>
+      <c r="C95" s="259" t="n"/>
+      <c r="D95" s="259" t="n"/>
+      <c r="E95" s="259" t="n"/>
+      <c r="F95" s="260" t="n"/>
+      <c r="G95" s="295" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº documento: </t>
+        </is>
+      </c>
+      <c r="H95" s="260" t="n"/>
+      <c r="I95" s="189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº documento: </t>
+        </is>
+      </c>
       <c r="J95" s="255" t="n"/>
       <c r="K95" s="255" t="n"/>
       <c r="L95" s="255" t="n"/>
       <c r="M95" s="255" t="n"/>
-      <c r="N95" s="255" t="n"/>
-      <c r="O95" s="255" t="n"/>
+      <c r="N95" s="256" t="n"/>
+      <c r="O95" s="189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nº do documento: </t>
+        </is>
+      </c>
       <c r="P95" s="255" t="n"/>
       <c r="Q95" s="255" t="n"/>
       <c r="R95" s="255" t="n"/>
       <c r="S95" s="255" t="n"/>
       <c r="T95" s="256" t="n"/>
     </row>
-    <row r="96" ht="34.9" customHeight="1">
-      <c r="B96" s="204" t="inlineStr">
-        <is>
-          <t>Declaro que fui treinado e que estou ciente dos riscos e exposições inerentes as atividades que irei executar conforme esta APR / DECLARAÇÃO DE MÉTODOS especificados neste documento.</t>
-        </is>
-      </c>
-      <c r="C96" s="255" t="n"/>
-      <c r="D96" s="255" t="n"/>
-      <c r="E96" s="255" t="n"/>
-      <c r="F96" s="255" t="n"/>
-      <c r="G96" s="255" t="n"/>
-      <c r="H96" s="255" t="n"/>
-      <c r="I96" s="255" t="n"/>
-      <c r="J96" s="255" t="n"/>
-      <c r="K96" s="255" t="n"/>
-      <c r="L96" s="255" t="n"/>
-      <c r="M96" s="255" t="n"/>
-      <c r="N96" s="255" t="n"/>
-      <c r="O96" s="255" t="n"/>
-      <c r="P96" s="255" t="n"/>
-      <c r="Q96" s="255" t="n"/>
-      <c r="R96" s="255" t="n"/>
-      <c r="S96" s="255" t="n"/>
-      <c r="T96" s="256" t="n"/>
-    </row>
-    <row r="97" ht="16.5" customHeight="1">
-      <c r="B97" s="145" t="inlineStr">
-        <is>
-          <t>NOME</t>
-        </is>
-      </c>
-      <c r="C97" s="255" t="n"/>
-      <c r="D97" s="255" t="n"/>
-      <c r="E97" s="256" t="n"/>
-      <c r="F97" s="145" t="inlineStr">
-        <is>
-          <t>CARGO</t>
-        </is>
-      </c>
-      <c r="G97" s="255" t="n"/>
+    <row r="96" ht="25.5" customHeight="1">
+      <c r="B96" s="294" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contato: </t>
+        </is>
+      </c>
+      <c r="C96" s="259" t="n"/>
+      <c r="D96" s="259" t="n"/>
+      <c r="E96" s="259" t="n"/>
+      <c r="F96" s="260" t="n"/>
+      <c r="G96" s="295" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contato: </t>
+        </is>
+      </c>
+      <c r="H96" s="260" t="n"/>
+      <c r="I96" s="296" t="inlineStr">
+        <is>
+          <t>Contato:</t>
+        </is>
+      </c>
+      <c r="J96" s="259" t="n"/>
+      <c r="K96" s="259" t="n"/>
+      <c r="L96" s="259" t="n"/>
+      <c r="M96" s="259" t="n"/>
+      <c r="N96" s="260" t="n"/>
+      <c r="O96" s="292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contato: </t>
+        </is>
+      </c>
+      <c r="P96" s="259" t="n"/>
+      <c r="Q96" s="259" t="n"/>
+      <c r="R96" s="259" t="n"/>
+      <c r="S96" s="259" t="n"/>
+      <c r="T96" s="293" t="n"/>
+    </row>
+    <row r="97" ht="42" customHeight="1">
+      <c r="B97" s="297" t="inlineStr">
+        <is>
+          <t>Assinatura:</t>
+        </is>
+      </c>
+      <c r="C97" s="259" t="n"/>
+      <c r="D97" s="259" t="n"/>
+      <c r="E97" s="259" t="n"/>
+      <c r="F97" s="260" t="n"/>
+      <c r="G97" s="186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assinatura:                                                       </t>
+        </is>
+      </c>
       <c r="H97" s="256" t="n"/>
-      <c r="I97" s="145" t="inlineStr">
-        <is>
-          <t>ASSINATURA</t>
+      <c r="I97" s="186" t="inlineStr">
+        <is>
+          <t>Assinatura:</t>
         </is>
       </c>
       <c r="J97" s="255" t="n"/>
       <c r="K97" s="255" t="n"/>
       <c r="L97" s="255" t="n"/>
       <c r="M97" s="255" t="n"/>
-      <c r="N97" s="255" t="n"/>
-      <c r="O97" s="255" t="n"/>
-      <c r="P97" s="256" t="n"/>
-      <c r="Q97" s="145" t="inlineStr">
-        <is>
-          <t>DATA</t>
-        </is>
-      </c>
-      <c r="R97" s="256" t="n"/>
-      <c r="S97" s="145" t="n"/>
+      <c r="N97" s="256" t="n"/>
+      <c r="O97" s="186" t="inlineStr">
+        <is>
+          <t>Assinatura:</t>
+        </is>
+      </c>
+      <c r="P97" s="255" t="n"/>
+      <c r="Q97" s="255" t="n"/>
+      <c r="R97" s="255" t="n"/>
+      <c r="S97" s="255" t="n"/>
       <c r="T97" s="256" t="n"/>
     </row>
-    <row r="98" ht="40.15" customHeight="1">
-      <c r="B98" s="144" t="n"/>
-      <c r="C98" s="255" t="n"/>
-      <c r="D98" s="255" t="n"/>
-      <c r="E98" s="256" t="n"/>
-      <c r="F98" s="144" t="n"/>
-      <c r="G98" s="255" t="n"/>
-      <c r="H98" s="256" t="n"/>
-      <c r="I98" s="144" t="n"/>
-      <c r="J98" s="255" t="n"/>
-      <c r="K98" s="255" t="n"/>
-      <c r="L98" s="255" t="n"/>
-      <c r="M98" s="255" t="n"/>
-      <c r="N98" s="255" t="n"/>
-      <c r="O98" s="255" t="n"/>
-      <c r="P98" s="256" t="n"/>
-      <c r="Q98" s="144" t="n"/>
-      <c r="R98" s="256" t="n"/>
-      <c r="S98" s="144" t="n"/>
-      <c r="T98" s="256" t="n"/>
-    </row>
-    <row r="99" ht="40.15" customHeight="1">
-      <c r="B99" s="144" t="n"/>
-      <c r="C99" s="255" t="n"/>
-      <c r="D99" s="255" t="n"/>
-      <c r="E99" s="256" t="n"/>
-      <c r="F99" s="144" t="n"/>
-      <c r="G99" s="255" t="n"/>
-      <c r="H99" s="256" t="n"/>
-      <c r="I99" s="144" t="n"/>
-      <c r="J99" s="255" t="n"/>
-      <c r="K99" s="255" t="n"/>
-      <c r="L99" s="255" t="n"/>
-      <c r="M99" s="255" t="n"/>
-      <c r="N99" s="255" t="n"/>
-      <c r="O99" s="255" t="n"/>
-      <c r="P99" s="256" t="n"/>
-      <c r="Q99" s="144" t="n"/>
-      <c r="R99" s="256" t="n"/>
-      <c r="S99" s="144" t="n"/>
-      <c r="T99" s="256" t="n"/>
-    </row>
-    <row r="100" ht="40.15" customHeight="1">
-      <c r="B100" s="144" t="n"/>
-      <c r="C100" s="255" t="n"/>
-      <c r="D100" s="255" t="n"/>
-      <c r="E100" s="256" t="n"/>
-      <c r="F100" s="144" t="n"/>
-      <c r="G100" s="255" t="n"/>
-      <c r="H100" s="256" t="n"/>
-      <c r="I100" s="144" t="n"/>
-      <c r="J100" s="255" t="n"/>
-      <c r="K100" s="255" t="n"/>
-      <c r="L100" s="255" t="n"/>
-      <c r="M100" s="255" t="n"/>
-      <c r="N100" s="255" t="n"/>
-      <c r="O100" s="255" t="n"/>
-      <c r="P100" s="256" t="n"/>
-      <c r="Q100" s="144" t="n"/>
-      <c r="R100" s="256" t="n"/>
-      <c r="S100" s="144" t="n"/>
-      <c r="T100" s="256" t="n"/>
-    </row>
-    <row r="101" ht="40.15" customHeight="1">
-      <c r="B101" s="144" t="n"/>
-      <c r="C101" s="255" t="n"/>
-      <c r="D101" s="255" t="n"/>
-      <c r="E101" s="256" t="n"/>
-      <c r="F101" s="144" t="n"/>
-      <c r="G101" s="255" t="n"/>
-      <c r="H101" s="256" t="n"/>
-      <c r="I101" s="144" t="n"/>
-      <c r="J101" s="255" t="n"/>
-      <c r="K101" s="255" t="n"/>
-      <c r="L101" s="255" t="n"/>
-      <c r="M101" s="255" t="n"/>
-      <c r="N101" s="255" t="n"/>
-      <c r="O101" s="255" t="n"/>
-      <c r="P101" s="256" t="n"/>
-      <c r="Q101" s="144" t="n"/>
-      <c r="R101" s="256" t="n"/>
-      <c r="S101" s="144" t="n"/>
-      <c r="T101" s="256" t="n"/>
-    </row>
-    <row r="102" ht="40.15" customHeight="1">
-      <c r="B102" s="144" t="n"/>
-      <c r="C102" s="255" t="n"/>
-      <c r="D102" s="255" t="n"/>
-      <c r="E102" s="256" t="n"/>
-      <c r="F102" s="144" t="n"/>
-      <c r="G102" s="255" t="n"/>
-      <c r="H102" s="256" t="n"/>
-      <c r="I102" s="144" t="n"/>
-      <c r="J102" s="255" t="n"/>
-      <c r="K102" s="255" t="n"/>
-      <c r="L102" s="255" t="n"/>
-      <c r="M102" s="255" t="n"/>
-      <c r="N102" s="255" t="n"/>
-      <c r="O102" s="255" t="n"/>
-      <c r="P102" s="256" t="n"/>
-      <c r="Q102" s="144" t="n"/>
-      <c r="R102" s="256" t="n"/>
-      <c r="S102" s="144" t="n"/>
-      <c r="T102" s="256" t="n"/>
-    </row>
-    <row r="103" ht="40.15" customHeight="1">
-      <c r="B103" s="144" t="n"/>
-      <c r="C103" s="255" t="n"/>
-      <c r="D103" s="255" t="n"/>
-      <c r="E103" s="256" t="n"/>
-      <c r="F103" s="144" t="n"/>
-      <c r="G103" s="255" t="n"/>
-      <c r="H103" s="256" t="n"/>
-      <c r="I103" s="144" t="n"/>
-      <c r="J103" s="255" t="n"/>
-      <c r="K103" s="255" t="n"/>
-      <c r="L103" s="255" t="n"/>
-      <c r="M103" s="255" t="n"/>
-      <c r="N103" s="255" t="n"/>
-      <c r="O103" s="255" t="n"/>
-      <c r="P103" s="256" t="n"/>
-      <c r="Q103" s="144" t="n"/>
-      <c r="R103" s="256" t="n"/>
-      <c r="S103" s="144" t="n"/>
-      <c r="T103" s="256" t="n"/>
-    </row>
-    <row r="104" ht="40.15" customHeight="1">
-      <c r="B104" s="144" t="n"/>
-      <c r="C104" s="255" t="n"/>
-      <c r="D104" s="255" t="n"/>
-      <c r="E104" s="256" t="n"/>
-      <c r="F104" s="144" t="n"/>
-      <c r="G104" s="255" t="n"/>
-      <c r="H104" s="256" t="n"/>
-      <c r="I104" s="144" t="n"/>
-      <c r="J104" s="255" t="n"/>
-      <c r="K104" s="255" t="n"/>
-      <c r="L104" s="255" t="n"/>
-      <c r="M104" s="255" t="n"/>
-      <c r="N104" s="255" t="n"/>
-      <c r="O104" s="255" t="n"/>
-      <c r="P104" s="256" t="n"/>
-      <c r="Q104" s="144" t="n"/>
-      <c r="R104" s="256" t="n"/>
-      <c r="S104" s="144" t="n"/>
-      <c r="T104" s="256" t="n"/>
-    </row>
-    <row r="105" ht="40.15" customHeight="1">
-      <c r="B105" s="144" t="n"/>
-      <c r="C105" s="255" t="n"/>
-      <c r="D105" s="255" t="n"/>
-      <c r="E105" s="256" t="n"/>
-      <c r="F105" s="144" t="n"/>
-      <c r="G105" s="255" t="n"/>
-      <c r="H105" s="256" t="n"/>
-      <c r="I105" s="144" t="n"/>
-      <c r="J105" s="255" t="n"/>
-      <c r="K105" s="255" t="n"/>
-      <c r="L105" s="255" t="n"/>
-      <c r="M105" s="255" t="n"/>
-      <c r="N105" s="255" t="n"/>
-      <c r="O105" s="255" t="n"/>
-      <c r="P105" s="256" t="n"/>
-      <c r="Q105" s="144" t="n"/>
-      <c r="R105" s="256" t="n"/>
-      <c r="S105" s="144" t="n"/>
-      <c r="T105" s="144" t="n"/>
-    </row>
-    <row r="106" ht="40.15" customHeight="1">
-      <c r="B106" s="144" t="n"/>
-      <c r="C106" s="255" t="n"/>
-      <c r="D106" s="255" t="n"/>
-      <c r="E106" s="256" t="n"/>
-      <c r="F106" s="144" t="n"/>
-      <c r="G106" s="255" t="n"/>
-      <c r="H106" s="256" t="n"/>
-      <c r="I106" s="144" t="n"/>
-      <c r="J106" s="255" t="n"/>
-      <c r="K106" s="255" t="n"/>
-      <c r="L106" s="255" t="n"/>
-      <c r="M106" s="255" t="n"/>
-      <c r="N106" s="255" t="n"/>
-      <c r="O106" s="255" t="n"/>
-      <c r="P106" s="256" t="n"/>
-      <c r="Q106" s="144" t="n"/>
-      <c r="R106" s="256" t="n"/>
-      <c r="S106" s="144" t="n"/>
-      <c r="T106" s="144" t="n"/>
-    </row>
-    <row r="107" ht="40.15" customHeight="1">
-      <c r="B107" s="144" t="n"/>
-      <c r="C107" s="255" t="n"/>
-      <c r="D107" s="255" t="n"/>
-      <c r="E107" s="256" t="n"/>
-      <c r="F107" s="144" t="n"/>
-      <c r="G107" s="255" t="n"/>
-      <c r="H107" s="256" t="n"/>
-      <c r="I107" s="144" t="n"/>
-      <c r="J107" s="255" t="n"/>
-      <c r="K107" s="255" t="n"/>
-      <c r="L107" s="255" t="n"/>
-      <c r="M107" s="255" t="n"/>
-      <c r="N107" s="255" t="n"/>
-      <c r="O107" s="255" t="n"/>
-      <c r="P107" s="256" t="n"/>
-      <c r="Q107" s="144" t="n"/>
-      <c r="R107" s="256" t="n"/>
-      <c r="S107" s="144" t="n"/>
-      <c r="T107" s="144" t="n"/>
-    </row>
-    <row r="108" ht="40.15" customHeight="1">
-      <c r="B108" s="144" t="n"/>
-      <c r="C108" s="255" t="n"/>
-      <c r="D108" s="255" t="n"/>
-      <c r="E108" s="256" t="n"/>
-      <c r="F108" s="144" t="n"/>
-      <c r="G108" s="255" t="n"/>
-      <c r="H108" s="256" t="n"/>
-      <c r="I108" s="144" t="n"/>
-      <c r="J108" s="255" t="n"/>
-      <c r="K108" s="255" t="n"/>
-      <c r="L108" s="255" t="n"/>
-      <c r="M108" s="255" t="n"/>
-      <c r="N108" s="255" t="n"/>
-      <c r="O108" s="255" t="n"/>
-      <c r="P108" s="256" t="n"/>
-      <c r="Q108" s="144" t="n"/>
-      <c r="R108" s="256" t="n"/>
-      <c r="S108" s="144" t="n"/>
-      <c r="T108" s="144" t="n"/>
-    </row>
-    <row r="109" ht="40.15" customHeight="1">
-      <c r="B109" s="144" t="n"/>
-      <c r="C109" s="255" t="n"/>
-      <c r="D109" s="255" t="n"/>
-      <c r="E109" s="256" t="n"/>
-      <c r="F109" s="144" t="n"/>
-      <c r="G109" s="255" t="n"/>
-      <c r="H109" s="256" t="n"/>
-      <c r="I109" s="144" t="n"/>
-      <c r="J109" s="255" t="n"/>
-      <c r="K109" s="255" t="n"/>
-      <c r="L109" s="255" t="n"/>
-      <c r="M109" s="255" t="n"/>
-      <c r="N109" s="255" t="n"/>
-      <c r="O109" s="255" t="n"/>
-      <c r="P109" s="256" t="n"/>
-      <c r="Q109" s="144" t="n"/>
-      <c r="R109" s="256" t="n"/>
-      <c r="S109" s="144" t="n"/>
-      <c r="T109" s="144" t="n"/>
-    </row>
-    <row r="110" ht="40.15" customHeight="1">
-      <c r="B110" s="144" t="n"/>
-      <c r="C110" s="255" t="n"/>
-      <c r="D110" s="255" t="n"/>
-      <c r="E110" s="256" t="n"/>
-      <c r="F110" s="144" t="n"/>
-      <c r="G110" s="255" t="n"/>
-      <c r="H110" s="256" t="n"/>
-      <c r="I110" s="144" t="n"/>
-      <c r="J110" s="255" t="n"/>
-      <c r="K110" s="255" t="n"/>
-      <c r="L110" s="255" t="n"/>
-      <c r="M110" s="255" t="n"/>
-      <c r="N110" s="255" t="n"/>
-      <c r="O110" s="255" t="n"/>
-      <c r="P110" s="256" t="n"/>
-      <c r="Q110" s="144" t="n"/>
-      <c r="R110" s="256" t="n"/>
-      <c r="S110" s="144" t="n"/>
-      <c r="T110" s="144" t="n"/>
-    </row>
-    <row r="111" ht="63.75" customHeight="1" thickBot="1">
-      <c r="B111" s="287" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL DA EMPRESA:</t>
-        </is>
-      </c>
-      <c r="C111" s="282" t="n"/>
-      <c r="D111" s="282" t="n"/>
-      <c r="E111" s="282" t="n"/>
-      <c r="F111" s="288" t="n"/>
-      <c r="G111" s="197" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL - SEGURANÇA DO TRABALHO EMPRESA</t>
-        </is>
-      </c>
-      <c r="H111" s="256" t="n"/>
-      <c r="I111" s="197" t="inlineStr">
-        <is>
-          <t>SEGURANÇA DO TRABALHO AMBEV</t>
-        </is>
-      </c>
-      <c r="J111" s="255" t="n"/>
-      <c r="K111" s="255" t="n"/>
-      <c r="L111" s="255" t="n"/>
-      <c r="M111" s="255" t="n"/>
-      <c r="N111" s="256" t="n"/>
-      <c r="O111" s="289" t="inlineStr">
-        <is>
-          <t>RESPONSÁVEL AMBEV PELA ATIVIDADE</t>
-        </is>
-      </c>
-      <c r="P111" s="282" t="n"/>
-      <c r="Q111" s="282" t="n"/>
-      <c r="R111" s="283" t="n"/>
-      <c r="S111" s="33" t="n"/>
-      <c r="T111" s="33" t="n"/>
-    </row>
-    <row r="112" ht="37.15" customHeight="1">
-      <c r="B112" s="290" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nome: </t>
-        </is>
-      </c>
-      <c r="C112" s="259" t="n"/>
-      <c r="D112" s="259" t="n"/>
-      <c r="E112" s="259" t="n"/>
-      <c r="F112" s="260" t="n"/>
-      <c r="G112" s="291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nome: </t>
-        </is>
-      </c>
-      <c r="H112" s="260" t="n"/>
-      <c r="I112" s="291" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nome: </t>
-        </is>
-      </c>
-      <c r="J112" s="259" t="n"/>
-      <c r="K112" s="259" t="n"/>
-      <c r="L112" s="259" t="n"/>
-      <c r="M112" s="259" t="n"/>
-      <c r="N112" s="260" t="n"/>
-      <c r="O112" s="292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nome: </t>
-        </is>
-      </c>
-      <c r="P112" s="259" t="n"/>
-      <c r="Q112" s="259" t="n"/>
-      <c r="R112" s="259" t="n"/>
-      <c r="S112" s="259" t="n"/>
-      <c r="T112" s="293" t="n"/>
-    </row>
-    <row r="113" ht="38.65" customHeight="1">
-      <c r="B113" s="294" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº documento: </t>
-        </is>
-      </c>
-      <c r="C113" s="259" t="n"/>
-      <c r="D113" s="259" t="n"/>
-      <c r="E113" s="259" t="n"/>
-      <c r="F113" s="260" t="n"/>
-      <c r="G113" s="295" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº documento: </t>
-        </is>
-      </c>
-      <c r="H113" s="260" t="n"/>
-      <c r="I113" s="189" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº documento: </t>
-        </is>
-      </c>
-      <c r="J113" s="255" t="n"/>
-      <c r="K113" s="255" t="n"/>
-      <c r="L113" s="255" t="n"/>
-      <c r="M113" s="255" t="n"/>
-      <c r="N113" s="256" t="n"/>
-      <c r="O113" s="189" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nº do documento: </t>
-        </is>
-      </c>
-      <c r="P113" s="255" t="n"/>
-      <c r="Q113" s="255" t="n"/>
-      <c r="R113" s="255" t="n"/>
-      <c r="S113" s="255" t="n"/>
-      <c r="T113" s="256" t="n"/>
-    </row>
-    <row r="114" ht="25.5" customHeight="1">
-      <c r="B114" s="294" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Contato: </t>
-        </is>
-      </c>
-      <c r="C114" s="259" t="n"/>
-      <c r="D114" s="259" t="n"/>
-      <c r="E114" s="259" t="n"/>
-      <c r="F114" s="260" t="n"/>
-      <c r="G114" s="295" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Contato: </t>
-        </is>
-      </c>
-      <c r="H114" s="260" t="n"/>
-      <c r="I114" s="296" t="inlineStr">
-        <is>
-          <t>Contato:</t>
-        </is>
-      </c>
-      <c r="J114" s="259" t="n"/>
-      <c r="K114" s="259" t="n"/>
-      <c r="L114" s="259" t="n"/>
-      <c r="M114" s="259" t="n"/>
-      <c r="N114" s="260" t="n"/>
-      <c r="O114" s="292" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Contato: </t>
-        </is>
-      </c>
-      <c r="P114" s="259" t="n"/>
-      <c r="Q114" s="259" t="n"/>
-      <c r="R114" s="259" t="n"/>
-      <c r="S114" s="259" t="n"/>
-      <c r="T114" s="293" t="n"/>
-    </row>
-    <row r="115" ht="42" customHeight="1">
-      <c r="B115" s="297" t="inlineStr">
-        <is>
-          <t>Assinatura:</t>
-        </is>
-      </c>
-      <c r="C115" s="259" t="n"/>
-      <c r="D115" s="259" t="n"/>
-      <c r="E115" s="259" t="n"/>
-      <c r="F115" s="260" t="n"/>
-      <c r="G115" s="186" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Assinatura:                                                       </t>
-        </is>
-      </c>
-      <c r="H115" s="256" t="n"/>
-      <c r="I115" s="186" t="inlineStr">
-        <is>
-          <t>Assinatura:</t>
-        </is>
-      </c>
-      <c r="J115" s="255" t="n"/>
-      <c r="K115" s="255" t="n"/>
-      <c r="L115" s="255" t="n"/>
-      <c r="M115" s="255" t="n"/>
-      <c r="N115" s="256" t="n"/>
-      <c r="O115" s="186" t="inlineStr">
-        <is>
-          <t>Assinatura:</t>
-        </is>
-      </c>
-      <c r="P115" s="255" t="n"/>
-      <c r="Q115" s="255" t="n"/>
-      <c r="R115" s="255" t="n"/>
-      <c r="S115" s="255" t="n"/>
-      <c r="T115" s="256" t="n"/>
-    </row>
+    <row r="98" ht="28.9" customHeight="1"/>
+    <row r="99" ht="26.45" customHeight="1"/>
+    <row r="100" ht="33" customHeight="1"/>
+    <row r="101" ht="18" customHeight="1"/>
+    <row r="102" ht="17.1" customHeight="1"/>
+    <row r="103" ht="17.1" customHeight="1"/>
+    <row r="104" ht="48.6" customHeight="1"/>
+    <row r="105" ht="362.25" customHeight="1"/>
+    <row r="106" ht="152.25" customHeight="1"/>
+    <row r="107" ht="47.25" customHeight="1"/>
+    <row r="108" ht="35.25" customHeight="1"/>
+    <row r="109" ht="28.5" customHeight="1"/>
+    <row r="110" ht="24.75" customHeight="1"/>
+    <row r="111" ht="24" customHeight="1" thickBot="1"/>
+    <row r="112" ht="21" customHeight="1"/>
+    <row r="113" ht="21" customHeight="1"/>
+    <row r="114" ht="17.1" customHeight="1"/>
+    <row r="115" ht="30" customHeight="1"/>
     <row r="116" ht="28.9" customHeight="1"/>
     <row r="117" ht="26.45" customHeight="1"/>
     <row r="118" ht="33" customHeight="1"/>
@@ -6007,341 +5400,291 @@
     <row r="228" ht="25.5" customHeight="1"/>
     <row r="229" ht="42" customHeight="1"/>
   </sheetData>
-  <mergeCells count="334">
+  <mergeCells count="284">
     <mergeCell ref="C47:D48"/>
-    <mergeCell ref="I105:P105"/>
+    <mergeCell ref="N76:O76"/>
     <mergeCell ref="F18:H18"/>
+    <mergeCell ref="K24:L24"/>
     <mergeCell ref="F33:H33"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="I115:N115"/>
-    <mergeCell ref="B68:E68"/>
+    <mergeCell ref="B74:E74"/>
+    <mergeCell ref="S81:T81"/>
+    <mergeCell ref="I93:N93"/>
     <mergeCell ref="P9:P12"/>
     <mergeCell ref="I4:L4"/>
-    <mergeCell ref="N94:O94"/>
     <mergeCell ref="I38:L38"/>
-    <mergeCell ref="O113:T113"/>
     <mergeCell ref="F17:H17"/>
-    <mergeCell ref="F100:H100"/>
-    <mergeCell ref="F109:H109"/>
-    <mergeCell ref="I101:P101"/>
+    <mergeCell ref="F66:H66"/>
+    <mergeCell ref="G97:H97"/>
     <mergeCell ref="M6:R6"/>
     <mergeCell ref="E61:F64"/>
     <mergeCell ref="B76:E76"/>
-    <mergeCell ref="M77:R77"/>
-    <mergeCell ref="B110:E110"/>
-    <mergeCell ref="Q79:Q82"/>
-    <mergeCell ref="I100:P100"/>
     <mergeCell ref="F31:H31"/>
-    <mergeCell ref="G65:G66"/>
-    <mergeCell ref="F102:H102"/>
+    <mergeCell ref="O95:T95"/>
     <mergeCell ref="Q26:Q29"/>
     <mergeCell ref="I30:O30"/>
     <mergeCell ref="P37:R37"/>
+    <mergeCell ref="Q88:R88"/>
     <mergeCell ref="F25:R25"/>
-    <mergeCell ref="I102:P102"/>
+    <mergeCell ref="E65:F65"/>
+    <mergeCell ref="Q90:R90"/>
     <mergeCell ref="G26:G29"/>
-    <mergeCell ref="Q99:R99"/>
     <mergeCell ref="B61:D64"/>
-    <mergeCell ref="S99:T99"/>
-    <mergeCell ref="G114:H114"/>
-    <mergeCell ref="Q110:R110"/>
+    <mergeCell ref="S83:T83"/>
     <mergeCell ref="B14:E14"/>
-    <mergeCell ref="O88:R88"/>
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="O35:R35"/>
-    <mergeCell ref="B78:E78"/>
-    <mergeCell ref="I65:O66"/>
+    <mergeCell ref="B69:E69"/>
+    <mergeCell ref="S85:T85"/>
     <mergeCell ref="B87:E87"/>
     <mergeCell ref="F21:H21"/>
-    <mergeCell ref="C83:D83"/>
     <mergeCell ref="E9:F12"/>
     <mergeCell ref="G43:G46"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="G61:G64"/>
-    <mergeCell ref="I104:P104"/>
+    <mergeCell ref="I66:N66"/>
     <mergeCell ref="F35:H35"/>
     <mergeCell ref="F50:H50"/>
     <mergeCell ref="I26:O29"/>
     <mergeCell ref="I53:N53"/>
-    <mergeCell ref="I68:N68"/>
-    <mergeCell ref="I106:P106"/>
-    <mergeCell ref="F89:R90"/>
     <mergeCell ref="F60:R60"/>
-    <mergeCell ref="Q102:R102"/>
     <mergeCell ref="F57:R57"/>
-    <mergeCell ref="G112:H112"/>
-    <mergeCell ref="N93:O93"/>
     <mergeCell ref="K41:L41"/>
     <mergeCell ref="B25:E25"/>
+    <mergeCell ref="O94:T94"/>
     <mergeCell ref="F41:J41"/>
     <mergeCell ref="O53:R53"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="I43:O46"/>
     <mergeCell ref="F49:H49"/>
     <mergeCell ref="P47:P48"/>
-    <mergeCell ref="S97:T97"/>
     <mergeCell ref="R47:R48"/>
     <mergeCell ref="B77:E77"/>
+    <mergeCell ref="Q89:R89"/>
     <mergeCell ref="P20:R20"/>
     <mergeCell ref="F69:H69"/>
-    <mergeCell ref="Q105:R105"/>
-    <mergeCell ref="F103:H103"/>
-    <mergeCell ref="I110:P110"/>
     <mergeCell ref="F42:R42"/>
     <mergeCell ref="O31:R31"/>
     <mergeCell ref="B53:E53"/>
     <mergeCell ref="I56:L56"/>
     <mergeCell ref="R61:R64"/>
-    <mergeCell ref="F75:R75"/>
-    <mergeCell ref="Q107:R107"/>
-    <mergeCell ref="Q104:R104"/>
+    <mergeCell ref="I70:N70"/>
     <mergeCell ref="F55:H55"/>
+    <mergeCell ref="Q91:R91"/>
     <mergeCell ref="B84:E84"/>
-    <mergeCell ref="Q100:R100"/>
-    <mergeCell ref="O71:R71"/>
-    <mergeCell ref="S100:T100"/>
-    <mergeCell ref="P79:P82"/>
-    <mergeCell ref="I112:N112"/>
-    <mergeCell ref="R79:R82"/>
+    <mergeCell ref="F73:G73"/>
     <mergeCell ref="P26:P29"/>
-    <mergeCell ref="Q106:R106"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="I61:O64"/>
-    <mergeCell ref="P94:T94"/>
     <mergeCell ref="B15:E15"/>
-    <mergeCell ref="I71:N71"/>
-    <mergeCell ref="O91:R91"/>
     <mergeCell ref="B24:E24"/>
-    <mergeCell ref="E83:F83"/>
-    <mergeCell ref="B95:E95"/>
+    <mergeCell ref="B80:E80"/>
+    <mergeCell ref="O73:R73"/>
     <mergeCell ref="M7:R7"/>
-    <mergeCell ref="S102:T102"/>
-    <mergeCell ref="I114:N114"/>
+    <mergeCell ref="B89:E89"/>
     <mergeCell ref="F38:H38"/>
     <mergeCell ref="B54:E56"/>
-    <mergeCell ref="B97:E97"/>
-    <mergeCell ref="F71:H71"/>
-    <mergeCell ref="F105:H105"/>
-    <mergeCell ref="S101:T101"/>
+    <mergeCell ref="S86:T86"/>
+    <mergeCell ref="B79:E79"/>
+    <mergeCell ref="O66:R66"/>
+    <mergeCell ref="C65:D65"/>
+    <mergeCell ref="I65:O65"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="F52:H52"/>
     <mergeCell ref="F67:H67"/>
+    <mergeCell ref="B81:E81"/>
     <mergeCell ref="K40:L40"/>
     <mergeCell ref="F37:H37"/>
     <mergeCell ref="E47:F48"/>
     <mergeCell ref="F54:R54"/>
-    <mergeCell ref="Q109:R109"/>
-    <mergeCell ref="F107:H107"/>
+    <mergeCell ref="F75:M75"/>
+    <mergeCell ref="F82:H82"/>
     <mergeCell ref="F23:J23"/>
-    <mergeCell ref="O115:T115"/>
-    <mergeCell ref="I107:P107"/>
+    <mergeCell ref="G95:H95"/>
     <mergeCell ref="F53:H53"/>
     <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B71:E73"/>
     <mergeCell ref="F58:J58"/>
+    <mergeCell ref="I83:P83"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="F68:H68"/>
-    <mergeCell ref="S104:T104"/>
     <mergeCell ref="F84:H84"/>
-    <mergeCell ref="P93:T93"/>
     <mergeCell ref="I9:O12"/>
     <mergeCell ref="B34:E34"/>
-    <mergeCell ref="E79:F82"/>
-    <mergeCell ref="B99:E99"/>
-    <mergeCell ref="B108:E108"/>
-    <mergeCell ref="B113:F113"/>
+    <mergeCell ref="F74:T74"/>
     <mergeCell ref="B47:B48"/>
+    <mergeCell ref="F80:H80"/>
+    <mergeCell ref="B83:E83"/>
+    <mergeCell ref="O70:R70"/>
     <mergeCell ref="B92:E92"/>
-    <mergeCell ref="I73:L73"/>
     <mergeCell ref="M40:R40"/>
     <mergeCell ref="B5:E5"/>
-    <mergeCell ref="B115:F115"/>
+    <mergeCell ref="B93:F93"/>
     <mergeCell ref="B85:E85"/>
-    <mergeCell ref="B94:E94"/>
     <mergeCell ref="M41:R41"/>
-    <mergeCell ref="F78:R78"/>
-    <mergeCell ref="I88:N88"/>
+    <mergeCell ref="F76:M76"/>
+    <mergeCell ref="I73:N73"/>
     <mergeCell ref="M24:R24"/>
-    <mergeCell ref="F92:T92"/>
     <mergeCell ref="K59:L59"/>
+    <mergeCell ref="I87:P87"/>
     <mergeCell ref="E30:F30"/>
-    <mergeCell ref="F73:H73"/>
     <mergeCell ref="F88:H88"/>
-    <mergeCell ref="B98:E98"/>
+    <mergeCell ref="I79:P79"/>
+    <mergeCell ref="I88:P88"/>
     <mergeCell ref="Q61:Q64"/>
+    <mergeCell ref="I82:P82"/>
+    <mergeCell ref="B95:F95"/>
     <mergeCell ref="I3:L3"/>
     <mergeCell ref="G47:G48"/>
-    <mergeCell ref="F74:H74"/>
     <mergeCell ref="I55:L55"/>
-    <mergeCell ref="I83:O83"/>
-    <mergeCell ref="F110:H110"/>
+    <mergeCell ref="F83:H83"/>
+    <mergeCell ref="B97:F97"/>
     <mergeCell ref="F85:H85"/>
-    <mergeCell ref="O67:R67"/>
     <mergeCell ref="F6:J6"/>
+    <mergeCell ref="N75:O75"/>
     <mergeCell ref="O14:R14"/>
     <mergeCell ref="H9:H12"/>
     <mergeCell ref="I67:N67"/>
-    <mergeCell ref="S98:T98"/>
+    <mergeCell ref="B91:E91"/>
     <mergeCell ref="I14:N14"/>
-    <mergeCell ref="K76:L76"/>
-    <mergeCell ref="B100:E100"/>
-    <mergeCell ref="F76:J76"/>
-    <mergeCell ref="B109:E109"/>
+    <mergeCell ref="F92:H92"/>
     <mergeCell ref="B22:E22"/>
     <mergeCell ref="K58:L58"/>
-    <mergeCell ref="B93:E93"/>
     <mergeCell ref="B31:E31"/>
-    <mergeCell ref="B102:E102"/>
+    <mergeCell ref="F77:T77"/>
     <mergeCell ref="F14:H14"/>
     <mergeCell ref="M23:R23"/>
     <mergeCell ref="H47:H48"/>
-    <mergeCell ref="H65:H66"/>
-    <mergeCell ref="B96:T96"/>
+    <mergeCell ref="I92:P92"/>
+    <mergeCell ref="B86:E86"/>
     <mergeCell ref="B39:E39"/>
     <mergeCell ref="B2:E4"/>
+    <mergeCell ref="O96:T96"/>
     <mergeCell ref="P55:R55"/>
     <mergeCell ref="F87:H87"/>
-    <mergeCell ref="B101:E101"/>
-    <mergeCell ref="F93:M93"/>
-    <mergeCell ref="G113:H113"/>
+    <mergeCell ref="O93:R93"/>
     <mergeCell ref="G9:G12"/>
-    <mergeCell ref="I79:O82"/>
-    <mergeCell ref="F72:R72"/>
+    <mergeCell ref="G94:H94"/>
+    <mergeCell ref="F89:H89"/>
+    <mergeCell ref="B94:F94"/>
     <mergeCell ref="F51:H51"/>
     <mergeCell ref="B40:E40"/>
     <mergeCell ref="B49:E49"/>
     <mergeCell ref="H26:H29"/>
-    <mergeCell ref="F95:T95"/>
+    <mergeCell ref="I81:P81"/>
+    <mergeCell ref="I90:P90"/>
     <mergeCell ref="I20:L20"/>
     <mergeCell ref="I18:N18"/>
-    <mergeCell ref="B79:D82"/>
-    <mergeCell ref="B104:E104"/>
-    <mergeCell ref="F101:H101"/>
     <mergeCell ref="B26:D29"/>
+    <mergeCell ref="F91:H91"/>
+    <mergeCell ref="B96:F96"/>
     <mergeCell ref="H43:H46"/>
     <mergeCell ref="B32:E32"/>
-    <mergeCell ref="Q97:R97"/>
     <mergeCell ref="F7:J7"/>
     <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B89:E91"/>
     <mergeCell ref="B35:E35"/>
     <mergeCell ref="B50:E50"/>
-    <mergeCell ref="B106:E106"/>
-    <mergeCell ref="O111:R111"/>
-    <mergeCell ref="B111:F111"/>
+    <mergeCell ref="I91:P91"/>
+    <mergeCell ref="I85:P85"/>
+    <mergeCell ref="B90:E90"/>
+    <mergeCell ref="Q79:R79"/>
     <mergeCell ref="P3:R3"/>
     <mergeCell ref="F19:R19"/>
-    <mergeCell ref="Q65:Q66"/>
-    <mergeCell ref="I84:N84"/>
+    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="I94:N94"/>
+    <mergeCell ref="Q81:R81"/>
     <mergeCell ref="B43:D46"/>
     <mergeCell ref="I31:N31"/>
+    <mergeCell ref="P75:T75"/>
     <mergeCell ref="F5:R5"/>
     <mergeCell ref="B67:E67"/>
     <mergeCell ref="I15:N15"/>
     <mergeCell ref="M59:R59"/>
     <mergeCell ref="R9:R12"/>
-    <mergeCell ref="F77:J77"/>
-    <mergeCell ref="I109:P109"/>
-    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="I95:N95"/>
+    <mergeCell ref="O97:T97"/>
     <mergeCell ref="K6:L6"/>
     <mergeCell ref="F3:H3"/>
     <mergeCell ref="F15:H15"/>
     <mergeCell ref="B19:E21"/>
     <mergeCell ref="F86:H86"/>
-    <mergeCell ref="F104:H104"/>
-    <mergeCell ref="G115:H115"/>
-    <mergeCell ref="I108:P108"/>
-    <mergeCell ref="P65:P66"/>
+    <mergeCell ref="I84:P84"/>
+    <mergeCell ref="F79:H79"/>
+    <mergeCell ref="I86:P86"/>
     <mergeCell ref="F32:H32"/>
-    <mergeCell ref="R65:R66"/>
-    <mergeCell ref="F97:H97"/>
-    <mergeCell ref="F106:H106"/>
+    <mergeCell ref="I80:P80"/>
+    <mergeCell ref="I89:P89"/>
     <mergeCell ref="Q43:Q46"/>
     <mergeCell ref="F40:J40"/>
+    <mergeCell ref="Q83:R83"/>
+    <mergeCell ref="F81:H81"/>
+    <mergeCell ref="Q92:R92"/>
+    <mergeCell ref="F90:H90"/>
     <mergeCell ref="F59:J59"/>
-    <mergeCell ref="I74:L74"/>
     <mergeCell ref="F24:J24"/>
-    <mergeCell ref="Q103:R103"/>
     <mergeCell ref="R26:R29"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="E26:F29"/>
-    <mergeCell ref="F94:M94"/>
+    <mergeCell ref="Q85:R85"/>
     <mergeCell ref="I35:N35"/>
-    <mergeCell ref="F91:G91"/>
-    <mergeCell ref="B71:E71"/>
-    <mergeCell ref="S103:T103"/>
-    <mergeCell ref="B105:E105"/>
     <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B72:E74"/>
     <mergeCell ref="B52:E52"/>
-    <mergeCell ref="Q98:R98"/>
+    <mergeCell ref="Q80:R80"/>
     <mergeCell ref="K23:L23"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="G79:G82"/>
+    <mergeCell ref="S80:T80"/>
+    <mergeCell ref="B60:E60"/>
     <mergeCell ref="I37:L37"/>
     <mergeCell ref="F34:H34"/>
-    <mergeCell ref="B60:E60"/>
     <mergeCell ref="F16:H16"/>
     <mergeCell ref="K7:L7"/>
     <mergeCell ref="F36:R36"/>
     <mergeCell ref="B57:E57"/>
     <mergeCell ref="P43:P46"/>
-    <mergeCell ref="F99:H99"/>
     <mergeCell ref="R43:R46"/>
-    <mergeCell ref="F108:H108"/>
     <mergeCell ref="I21:L21"/>
     <mergeCell ref="F8:R8"/>
-    <mergeCell ref="B114:F114"/>
     <mergeCell ref="F2:R2"/>
-    <mergeCell ref="I99:P99"/>
     <mergeCell ref="B9:D12"/>
+    <mergeCell ref="B78:T78"/>
+    <mergeCell ref="G96:H96"/>
     <mergeCell ref="F20:H20"/>
-    <mergeCell ref="E65:F66"/>
+    <mergeCell ref="Q87:R87"/>
     <mergeCell ref="F22:R22"/>
     <mergeCell ref="I32:N32"/>
-    <mergeCell ref="O112:T112"/>
+    <mergeCell ref="I97:N97"/>
+    <mergeCell ref="P76:T76"/>
     <mergeCell ref="F70:H70"/>
     <mergeCell ref="F39:R39"/>
-    <mergeCell ref="O114:T114"/>
+    <mergeCell ref="I96:N96"/>
     <mergeCell ref="I13:O13"/>
     <mergeCell ref="B36:E38"/>
-    <mergeCell ref="I111:N111"/>
+    <mergeCell ref="Q82:R82"/>
     <mergeCell ref="B75:E75"/>
     <mergeCell ref="I47:O48"/>
     <mergeCell ref="P61:P64"/>
-    <mergeCell ref="H79:H82"/>
+    <mergeCell ref="S82:T82"/>
     <mergeCell ref="H61:H64"/>
     <mergeCell ref="F56:H56"/>
-    <mergeCell ref="I103:P103"/>
     <mergeCell ref="B59:E59"/>
-    <mergeCell ref="I97:P97"/>
+    <mergeCell ref="G93:H93"/>
     <mergeCell ref="O18:R18"/>
-    <mergeCell ref="M76:R76"/>
     <mergeCell ref="Q9:Q12"/>
-    <mergeCell ref="B65:B66"/>
-    <mergeCell ref="K77:L77"/>
-    <mergeCell ref="F98:H98"/>
     <mergeCell ref="I50:N50"/>
     <mergeCell ref="B70:E70"/>
-    <mergeCell ref="B112:F112"/>
+    <mergeCell ref="F71:R72"/>
+    <mergeCell ref="Q84:R84"/>
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="M58:R58"/>
     <mergeCell ref="O49:R49"/>
-    <mergeCell ref="I98:P98"/>
+    <mergeCell ref="S84:T84"/>
     <mergeCell ref="E43:F46"/>
-    <mergeCell ref="P73:R73"/>
-    <mergeCell ref="G111:H111"/>
-    <mergeCell ref="Q108:R108"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="I49:N49"/>
-    <mergeCell ref="O84:R84"/>
+    <mergeCell ref="Q86:R86"/>
     <mergeCell ref="B88:E88"/>
+    <mergeCell ref="B82:E82"/>
     <mergeCell ref="Q47:Q48"/>
-    <mergeCell ref="Q101:R101"/>
     <mergeCell ref="C13:D13"/>
-    <mergeCell ref="I113:N113"/>
-    <mergeCell ref="I91:N91"/>
-    <mergeCell ref="I85:N85"/>
-    <mergeCell ref="C65:D66"/>
+    <mergeCell ref="S79:T79"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.2362204724409449" right="0.2362204724409449" top="0.7480314960629921" bottom="0.7480314960629921" header="0.3149606299212598" footer="0.3149606299212598"/>
@@ -6354,13 +5697,12 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <rowBreaks count="6" manualBreakCount="6">
+  <rowBreaks count="5" manualBreakCount="5">
     <brk id="18" min="0" max="16383" man="1"/>
     <brk id="35" min="0" max="16383" man="1"/>
     <brk id="53" min="0" max="16383" man="1"/>
-    <brk id="71" min="0" max="16383" man="1"/>
-    <brk id="88" min="0" max="16383" man="1"/>
-    <brk id="115" min="0" max="16383" man="1"/>
+    <brk id="70" min="0" max="16383" man="1"/>
+    <brk id="97" min="0" max="16383" man="1"/>
   </rowBreaks>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>

</xml_diff>